<commit_message>
docs(limet): Q-20 ciclo di rilavorazione code review (H-716, T-716, E2E-REV-1), xlsx a 80 task
</commit_message>
<xml_diff>
--- a/log/HELIOS_Distribuzione_task.xlsx
+++ b/log/HELIOS_Distribuzione_task.xlsx
@@ -16,8 +16,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pre-GO'!$A$4:$V$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Post-GO'!$A$4:$V$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pacchetti'!$A$4:$N$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Post-GO'!$A$4:$V$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pacchetti'!$A$4:$N$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -639,7 +639,7 @@
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIF('Post-GO'!I5:I61,A4)</f>
+        <f>COUNTIF('Post-GO'!I5:I62,A4)</f>
         <v/>
       </c>
       <c r="D4">
@@ -658,7 +658,7 @@
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIF('Post-GO'!I5:I61,A5)</f>
+        <f>COUNTIF('Post-GO'!I5:I62,A5)</f>
         <v/>
       </c>
       <c r="D5">
@@ -677,7 +677,7 @@
         <v/>
       </c>
       <c r="C6">
-        <f>COUNTIF('Post-GO'!I5:I61,A6)</f>
+        <f>COUNTIF('Post-GO'!I5:I62,A6)</f>
         <v/>
       </c>
       <c r="D6">
@@ -696,7 +696,7 @@
         <v/>
       </c>
       <c r="C7">
-        <f>COUNTIF('Post-GO'!I5:I61,A7)</f>
+        <f>COUNTIF('Post-GO'!I5:I62,A7)</f>
         <v/>
       </c>
       <c r="D7">
@@ -715,7 +715,7 @@
         <v/>
       </c>
       <c r="C8">
-        <f>COUNTIF('Post-GO'!I5:I61,A8)</f>
+        <f>COUNTIF('Post-GO'!I5:I62,A8)</f>
         <v/>
       </c>
       <c r="D8">
@@ -799,7 +799,7 @@
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIF('Post-GO'!K5:K61,A14)</f>
+        <f>COUNTIF('Post-GO'!K5:K62,A14)</f>
         <v/>
       </c>
       <c r="D14">
@@ -807,7 +807,7 @@
         <v/>
       </c>
       <c r="E14">
-        <f>COUNTIFS('Pre-GO'!K5:K26,A14,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!K5:K61,A14,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!K5:K26,A14,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!K5:K62,A14,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
     </row>
@@ -822,7 +822,7 @@
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIF('Post-GO'!K5:K61,A15)</f>
+        <f>COUNTIF('Post-GO'!K5:K62,A15)</f>
         <v/>
       </c>
       <c r="D15">
@@ -830,7 +830,7 @@
         <v/>
       </c>
       <c r="E15">
-        <f>COUNTIFS('Pre-GO'!K5:K26,A15,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!K5:K61,A15,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!K5:K26,A15,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!K5:K62,A15,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
     </row>
@@ -845,7 +845,7 @@
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIF('Post-GO'!K5:K61,A16)</f>
+        <f>COUNTIF('Post-GO'!K5:K62,A16)</f>
         <v/>
       </c>
       <c r="D16">
@@ -853,7 +853,7 @@
         <v/>
       </c>
       <c r="E16">
-        <f>COUNTIFS('Pre-GO'!K5:K26,A16,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!K5:K61,A16,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!K5:K26,A16,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!K5:K62,A16,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
     </row>
@@ -868,7 +868,7 @@
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIF('Post-GO'!K5:K61,A17)</f>
+        <f>COUNTIF('Post-GO'!K5:K62,A17)</f>
         <v/>
       </c>
       <c r="D17">
@@ -876,7 +876,7 @@
         <v/>
       </c>
       <c r="E17">
-        <f>COUNTIFS('Pre-GO'!K5:K26,A17,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!K5:K61,A17,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!K5:K26,A17,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!K5:K62,A17,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
     </row>
@@ -919,19 +919,19 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-00")+COUNTIF('Post-GO'!D5:D61,"PK-00")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-00")+COUNTIF('Post-GO'!D5:D62,"PK-00")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-00",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-00",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-00",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-00",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D21">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-00",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-00",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-00",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-00",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E21">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-00",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-00",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-00",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-00",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F21" s="5">
@@ -946,19 +946,19 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-01")+COUNTIF('Post-GO'!D5:D61,"PK-01")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-01")+COUNTIF('Post-GO'!D5:D62,"PK-01")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-01",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-01",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-01",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-01",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D22">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-01",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-01",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-01",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-01",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E22">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-01",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-01",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-01",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-01",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F22" s="5">
@@ -973,19 +973,19 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-02")+COUNTIF('Post-GO'!D5:D61,"PK-02")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-02")+COUNTIF('Post-GO'!D5:D62,"PK-02")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-02",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-02",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-02",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-02",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D23">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-02",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-02",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-02",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-02",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E23">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-02",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-02",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-02",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-02",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F23" s="5">
@@ -1000,19 +1000,19 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-03")+COUNTIF('Post-GO'!D5:D61,"PK-03")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-03")+COUNTIF('Post-GO'!D5:D62,"PK-03")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-03",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-03",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-03",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-03",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D24">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-03",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-03",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-03",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-03",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E24">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-03",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-03",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-03",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-03",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F24" s="5">
@@ -1027,19 +1027,19 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-04")+COUNTIF('Post-GO'!D5:D61,"PK-04")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-04")+COUNTIF('Post-GO'!D5:D62,"PK-04")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-04",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-04",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-04",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-04",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D25">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-04",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-04",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-04",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-04",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E25">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-04",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-04",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-04",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-04",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F25" s="5">
@@ -1054,19 +1054,19 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-05")+COUNTIF('Post-GO'!D5:D61,"PK-05")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-05")+COUNTIF('Post-GO'!D5:D62,"PK-05")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-05",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-05",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D26">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-05",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-05",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E26">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-05",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-05",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F26" s="5">
@@ -1081,19 +1081,19 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-05b")+COUNTIF('Post-GO'!D5:D61,"PK-05b")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-05b")+COUNTIF('Post-GO'!D5:D62,"PK-05b")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-05b",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-05b",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D27">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-05b",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-05b",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E27">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-05b",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-05b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-05b",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F27" s="5">
@@ -1108,19 +1108,19 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-06")+COUNTIF('Post-GO'!D5:D61,"PK-06")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-06")+COUNTIF('Post-GO'!D5:D62,"PK-06")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-06",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-06",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-06",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-06",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D28">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-06",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-06",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-06",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-06",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E28">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-06",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-06",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-06",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-06",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F28" s="5">
@@ -1135,19 +1135,19 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-07")+COUNTIF('Post-GO'!D5:D61,"PK-07")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-07")+COUNTIF('Post-GO'!D5:D62,"PK-07")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-07",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-07",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D29">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-07",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-07",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E29">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-07",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-07",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F29" s="5">
@@ -1162,19 +1162,19 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-07b")+COUNTIF('Post-GO'!D5:D61,"PK-07b")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-07b")+COUNTIF('Post-GO'!D5:D62,"PK-07b")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-07b",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-07b",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D30">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-07b",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-07b",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E30">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-07b",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-07b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-07b",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F30" s="5">
@@ -1189,19 +1189,19 @@
         </is>
       </c>
       <c r="B31">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-08")+COUNTIF('Post-GO'!D5:D61,"PK-08")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-08")+COUNTIF('Post-GO'!D5:D62,"PK-08")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-08",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-08",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-08",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-08",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D31">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-08",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-08",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-08",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-08",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E31">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-08",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-08",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-08",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-08",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F31" s="5">
@@ -1216,19 +1216,19 @@
         </is>
       </c>
       <c r="B32">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-09")+COUNTIF('Post-GO'!D5:D61,"PK-09")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-09")+COUNTIF('Post-GO'!D5:D62,"PK-09")</f>
         <v/>
       </c>
       <c r="C32">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-09",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-09",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-09",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-09",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D32">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-09",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-09",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-09",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-09",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E32">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-09",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-09",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-09",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-09",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F32" s="5">
@@ -1243,19 +1243,19 @@
         </is>
       </c>
       <c r="B33">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-10")+COUNTIF('Post-GO'!D5:D61,"PK-10")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-10")+COUNTIF('Post-GO'!D5:D62,"PK-10")</f>
         <v/>
       </c>
       <c r="C33">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-10",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-10",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-10",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-10",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D33">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-10",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-10",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-10",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-10",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E33">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-10",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-10",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-10",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-10",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F33" s="5">
@@ -1270,19 +1270,19 @@
         </is>
       </c>
       <c r="B34">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-11")+COUNTIF('Post-GO'!D5:D61,"PK-11")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-11")+COUNTIF('Post-GO'!D5:D62,"PK-11")</f>
         <v/>
       </c>
       <c r="C34">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-11",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-11",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-11",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-11",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D34">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-11",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-11",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-11",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-11",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E34">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-11",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-11",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-11",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-11",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F34" s="5">
@@ -1297,19 +1297,19 @@
         </is>
       </c>
       <c r="B35">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-12")+COUNTIF('Post-GO'!D5:D61,"PK-12")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-12")+COUNTIF('Post-GO'!D5:D62,"PK-12")</f>
         <v/>
       </c>
       <c r="C35">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-12",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-12",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-12",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-12",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D35">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-12",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-12",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-12",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-12",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E35">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-12",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-12",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-12",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-12",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F35" s="5">
@@ -1324,19 +1324,19 @@
         </is>
       </c>
       <c r="B36">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-13")+COUNTIF('Post-GO'!D5:D61,"PK-13")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-13")+COUNTIF('Post-GO'!D5:D62,"PK-13")</f>
         <v/>
       </c>
       <c r="C36">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-13",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-13",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-13",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-13",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D36">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-13",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-13",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-13",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-13",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E36">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-13",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-13",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-13",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-13",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F36" s="5">
@@ -1351,19 +1351,19 @@
         </is>
       </c>
       <c r="B37">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-14")+COUNTIF('Post-GO'!D5:D61,"PK-14")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-14")+COUNTIF('Post-GO'!D5:D62,"PK-14")</f>
         <v/>
       </c>
       <c r="C37">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-14",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-14",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-14",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-14",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D37">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-14",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-14",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-14",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-14",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E37">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-14",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-14",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-14",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-14",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F37" s="5">
@@ -1378,19 +1378,19 @@
         </is>
       </c>
       <c r="B38">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-15")+COUNTIF('Post-GO'!D5:D61,"PK-15")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-15")+COUNTIF('Post-GO'!D5:D62,"PK-15")</f>
         <v/>
       </c>
       <c r="C38">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-15",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-15",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-15",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-15",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D38">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-15",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-15",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-15",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-15",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E38">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-15",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-15",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-15",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-15",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F38" s="5">
@@ -1405,19 +1405,19 @@
         </is>
       </c>
       <c r="B39">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-16")+COUNTIF('Post-GO'!D5:D61,"PK-16")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-16")+COUNTIF('Post-GO'!D5:D62,"PK-16")</f>
         <v/>
       </c>
       <c r="C39">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-16",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-16",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D39">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-16",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-16",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E39">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-16",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-16",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F39" s="5">
@@ -1432,19 +1432,19 @@
         </is>
       </c>
       <c r="B40">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-16b")+COUNTIF('Post-GO'!D5:D61,"PK-16b")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-16b")+COUNTIF('Post-GO'!D5:D62,"PK-16b")</f>
         <v/>
       </c>
       <c r="C40">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-16b",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-16b",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D40">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-16b",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-16b",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E40">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-16b",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-16b",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F40" s="5">
@@ -1459,19 +1459,19 @@
         </is>
       </c>
       <c r="B41">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-16c")+COUNTIF('Post-GO'!D5:D61,"PK-16c")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-16c")+COUNTIF('Post-GO'!D5:D62,"PK-16c")</f>
         <v/>
       </c>
       <c r="C41">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16c",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-16c",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16c",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-16c",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D41">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16c",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-16c",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16c",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-16c",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E41">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16c",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-16c",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-16c",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-16c",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F41" s="5">
@@ -1486,19 +1486,19 @@
         </is>
       </c>
       <c r="B42">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-17")+COUNTIF('Post-GO'!D5:D61,"PK-17")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-17")+COUNTIF('Post-GO'!D5:D62,"PK-17")</f>
         <v/>
       </c>
       <c r="C42">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-17",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-17",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-17",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-17",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D42">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-17",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-17",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-17",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-17",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E42">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-17",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-17",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-17",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-17",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F42" s="5">
@@ -1513,19 +1513,19 @@
         </is>
       </c>
       <c r="B43">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-18")+COUNTIF('Post-GO'!D5:D61,"PK-18")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-18")+COUNTIF('Post-GO'!D5:D62,"PK-18")</f>
         <v/>
       </c>
       <c r="C43">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-18",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-18",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-18",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-18",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D43">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-18",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-18",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-18",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-18",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E43">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-18",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-18",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-18",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-18",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F43" s="5">
@@ -1540,19 +1540,19 @@
         </is>
       </c>
       <c r="B44">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-19")+COUNTIF('Post-GO'!D5:D61,"PK-19")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-19")+COUNTIF('Post-GO'!D5:D62,"PK-19")</f>
         <v/>
       </c>
       <c r="C44">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-19",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-19",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D44">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-19",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-19",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E44">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-19",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-19",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F44" s="5">
@@ -1567,19 +1567,19 @@
         </is>
       </c>
       <c r="B45">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-20")+COUNTIF('Post-GO'!D5:D61,"PK-20")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-20")+COUNTIF('Post-GO'!D5:D62,"PK-20")</f>
         <v/>
       </c>
       <c r="C45">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-20",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-20",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D45">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-20",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-20",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E45">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-20",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-20",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F45" s="5">
@@ -1594,19 +1594,19 @@
         </is>
       </c>
       <c r="B46">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-19b")+COUNTIF('Post-GO'!D5:D61,"PK-19b")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-19b")+COUNTIF('Post-GO'!D5:D62,"PK-19b")</f>
         <v/>
       </c>
       <c r="C46">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-19b",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-19b",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D46">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-19b",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-19b",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E46">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-19b",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-19b",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F46" s="5">
@@ -1621,19 +1621,19 @@
         </is>
       </c>
       <c r="B47">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-20b")+COUNTIF('Post-GO'!D5:D61,"PK-20b")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-20b")+COUNTIF('Post-GO'!D5:D62,"PK-20b")</f>
         <v/>
       </c>
       <c r="C47">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-20b",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-20b",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D47">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-20b",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-20b",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E47">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-20b",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-20b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-20b",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F47" s="5">
@@ -1644,23 +1644,23 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PK-21 · Valutazione rischi di prodotto (C28)</t>
+          <t>PK-19c · Ciclo di rilavorazione dei findings di code review</t>
         </is>
       </c>
       <c r="B48">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-21")+COUNTIF('Post-GO'!D5:D61,"PK-21")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-19c")+COUNTIF('Post-GO'!D5:D62,"PK-19c")</f>
         <v/>
       </c>
       <c r="C48">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-21",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-21",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19c",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-19c",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D48">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-21",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-21",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19c",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-19c",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E48">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-21",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-21",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-19c",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-19c",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F48" s="5">
@@ -1671,23 +1671,23 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PK-22 · Installer e modifiche documentali a LIMET</t>
+          <t>PK-21 · Valutazione rischi di prodotto (C28)</t>
         </is>
       </c>
       <c r="B49">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-22")+COUNTIF('Post-GO'!D5:D61,"PK-22")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-21")+COUNTIF('Post-GO'!D5:D62,"PK-21")</f>
         <v/>
       </c>
       <c r="C49">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-22",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-22",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-21",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-21",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D49">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-22",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-22",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-21",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-21",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E49">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-22",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-22",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-21",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-21",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F49" s="5">
@@ -1698,23 +1698,23 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PK-23 · Hook ECC e registro chiamate LLM</t>
+          <t>PK-22 · Installer e modifiche documentali a LIMET</t>
         </is>
       </c>
       <c r="B50">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-23")+COUNTIF('Post-GO'!D5:D61,"PK-23")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-22")+COUNTIF('Post-GO'!D5:D62,"PK-22")</f>
         <v/>
       </c>
       <c r="C50">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-23",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-23",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-22",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-22",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D50">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-23",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-23",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-22",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-22",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E50">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-23",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-23",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-22",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-22",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F50" s="5">
@@ -1725,23 +1725,23 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PK-24 · Knowledge base HLS_* e accesso agenti</t>
+          <t>PK-23 · Hook ECC e registro chiamate LLM</t>
         </is>
       </c>
       <c r="B51">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-24")+COUNTIF('Post-GO'!D5:D61,"PK-24")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-23")+COUNTIF('Post-GO'!D5:D62,"PK-23")</f>
         <v/>
       </c>
       <c r="C51">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-24",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-24",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-23",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-23",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D51">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-24",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-24",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-23",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-23",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E51">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-24",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-24",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-23",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-23",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F51" s="5">
@@ -1752,23 +1752,23 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PK-25 · API loopback e read model</t>
+          <t>PK-24 · Knowledge base HLS_* e accesso agenti</t>
         </is>
       </c>
       <c r="B52">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-25")+COUNTIF('Post-GO'!D5:D61,"PK-25")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-24")+COUNTIF('Post-GO'!D5:D62,"PK-24")</f>
         <v/>
       </c>
       <c r="C52">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-25",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-25",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-24",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-24",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D52">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-25",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-25",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-24",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-24",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E52">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-25",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-25",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-24",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-24",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F52" s="5">
@@ -1779,23 +1779,23 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PK-26 · UI (viste, permessi, grafica, npm) e sostituzione launcher</t>
+          <t>PK-25 · API loopback e read model</t>
         </is>
       </c>
       <c r="B53">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-26")+COUNTIF('Post-GO'!D5:D61,"PK-26")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-25")+COUNTIF('Post-GO'!D5:D62,"PK-25")</f>
         <v/>
       </c>
       <c r="C53">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-26",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-25",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-25",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D53">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-26",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-25",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-25",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E53">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-26",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-25",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-25",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F53" s="5">
@@ -1806,23 +1806,23 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PK-26b · Gate di configurazione all'avvio della dashboard</t>
+          <t>PK-26 · UI (viste, permessi, grafica, npm) e sostituzione launcher</t>
         </is>
       </c>
       <c r="B54">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-26b")+COUNTIF('Post-GO'!D5:D61,"PK-26b")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-26")+COUNTIF('Post-GO'!D5:D62,"PK-26")</f>
         <v/>
       </c>
       <c r="C54">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-26b",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-26",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D54">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-26b",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-26",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E54">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-26b",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-26",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F54" s="5">
@@ -1833,23 +1833,23 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PK-26c · Pannello di avvio del run non presidiato</t>
+          <t>PK-26b · Gate di configurazione all'avvio della dashboard</t>
         </is>
       </c>
       <c r="B55">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-26c")+COUNTIF('Post-GO'!D5:D61,"PK-26c")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-26b")+COUNTIF('Post-GO'!D5:D62,"PK-26b")</f>
         <v/>
       </c>
       <c r="C55">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26c",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-26c",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26b",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-26b",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D55">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26c",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-26c",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26b",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-26b",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E55">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26c",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-26c",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26b",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-26b",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F55" s="5">
@@ -1860,23 +1860,23 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PK-27 · Scenari E2E V1–V24</t>
+          <t>PK-26c · Pannello di avvio del run non presidiato</t>
         </is>
       </c>
       <c r="B56">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-27")+COUNTIF('Post-GO'!D5:D61,"PK-27")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-26c")+COUNTIF('Post-GO'!D5:D62,"PK-26c")</f>
         <v/>
       </c>
       <c r="C56">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-27",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-27",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26c",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-26c",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D56">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-27",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-27",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26c",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-26c",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E56">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-27",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-27",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-26c",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-26c",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F56" s="5">
@@ -1887,23 +1887,23 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PK-28 · README plugin e manuali</t>
+          <t>PK-27 · Scenari E2E V1–V24</t>
         </is>
       </c>
       <c r="B57">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-28")+COUNTIF('Post-GO'!D5:D61,"PK-28")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-27")+COUNTIF('Post-GO'!D5:D62,"PK-27")</f>
         <v/>
       </c>
       <c r="C57">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-28",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-28",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-27",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-27",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D57">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-28",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-28",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-27",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-27",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E57">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-28",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-28",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-27",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-27",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F57" s="5">
@@ -1914,23 +1914,23 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PK-29 · Hardening</t>
+          <t>PK-28 · README plugin e manuali</t>
         </is>
       </c>
       <c r="B58">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-29")+COUNTIF('Post-GO'!D5:D61,"PK-29")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-28")+COUNTIF('Post-GO'!D5:D62,"PK-28")</f>
         <v/>
       </c>
       <c r="C58">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-29",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-29",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-28",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-28",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D58">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-29",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-29",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-28",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-28",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E58">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-29",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-29",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-28",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-28",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F58" s="5">
@@ -1941,23 +1941,23 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PK-30 · Rollout sul pilota</t>
+          <t>PK-29 · Hardening</t>
         </is>
       </c>
       <c r="B59">
-        <f>COUNTIF('Pre-GO'!D5:D26,"PK-30")+COUNTIF('Post-GO'!D5:D61,"PK-30")</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-29")+COUNTIF('Post-GO'!D5:D62,"PK-29")</f>
         <v/>
       </c>
       <c r="C59">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-30",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,"PK-30",'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-29",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-29",'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D59">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-30",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,"PK-30",'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-29",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-29",'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E59">
-        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-30",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D61,"PK-30",'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-29",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-29",'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F59" s="5">
@@ -1965,88 +1965,90 @@
         <v/>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="6" t="inlineStr">
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>PK-30 · Rollout sul pilota</t>
+        </is>
+      </c>
+      <c r="B60">
+        <f>COUNTIF('Pre-GO'!D5:D26,"PK-30")+COUNTIF('Post-GO'!D5:D62,"PK-30")</f>
+        <v/>
+      </c>
+      <c r="C60">
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-30",'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,"PK-30",'Post-GO'!I5:I62,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="D60">
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-30",'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,"PK-30",'Post-GO'!I5:I62,"In corso")</f>
+        <v/>
+      </c>
+      <c r="E60">
+        <f>COUNTIFS('Pre-GO'!D5:D26,"PK-30",'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!D5:D62,"PK-30",'Post-GO'!I5:I62,"Da fare")</f>
+        <v/>
+      </c>
+      <c r="F60" s="5">
+        <f>IF(B60=0,0,C60/B60)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>Avanzamento per fase</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Fatti</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>In corso</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>Da fare</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B63">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A63)+COUNTIFS('Post-GO'!A5:A61,$A63)</f>
-        <v/>
-      </c>
-      <c r="C63">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A63,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A63,'Post-GO'!I5:I61,"Fatto")</f>
-        <v/>
-      </c>
-      <c r="D63">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A63,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A63,'Post-GO'!I5:I61,"In corso")</f>
-        <v/>
-      </c>
-      <c r="E63">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A63,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A63,'Post-GO'!I5:I61,"Da fare")</f>
-        <v/>
-      </c>
-      <c r="F63" s="5">
-        <f>IF(B63=0,0,C63/B63)</f>
-        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B64">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A64)+COUNTIFS('Post-GO'!A5:A61,$A64)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A64)+COUNTIFS('Post-GO'!A5:A62,$A64)</f>
         <v/>
       </c>
       <c r="C64">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A64,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A64,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A64,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A64,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D64">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A64,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A64,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A64,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A64,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E64">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A64,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A64,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A64,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A64,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F64" s="5">
@@ -2056,22 +2058,22 @@
     </row>
     <row r="65">
       <c r="A65" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B65">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A65)+COUNTIFS('Post-GO'!A5:A61,$A65)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A65)+COUNTIFS('Post-GO'!A5:A62,$A65)</f>
         <v/>
       </c>
       <c r="C65">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A65,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A65,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A65,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A65,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D65">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A65,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A65,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A65,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A65,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E65">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A65,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A65,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A65,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A65,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F65" s="5">
@@ -2081,22 +2083,22 @@
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B66">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A66)+COUNTIFS('Post-GO'!A5:A61,$A66)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A66)+COUNTIFS('Post-GO'!A5:A62,$A66)</f>
         <v/>
       </c>
       <c r="C66">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A66,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A66,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A66,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A66,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D66">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A66,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A66,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A66,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A66,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E66">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A66,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A66,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A66,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A66,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F66" s="5">
@@ -2106,22 +2108,22 @@
     </row>
     <row r="67">
       <c r="A67" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B67">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A67)+COUNTIFS('Post-GO'!A5:A61,$A67)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A67)+COUNTIFS('Post-GO'!A5:A62,$A67)</f>
         <v/>
       </c>
       <c r="C67">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A67,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A67,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A67,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A67,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D67">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A67,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A67,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A67,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A67,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E67">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A67,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A67,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A67,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A67,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F67" s="5">
@@ -2131,22 +2133,22 @@
     </row>
     <row r="68">
       <c r="A68" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B68">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A68)+COUNTIFS('Post-GO'!A5:A61,$A68)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A68)+COUNTIFS('Post-GO'!A5:A62,$A68)</f>
         <v/>
       </c>
       <c r="C68">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A68,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A68,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A68,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A68,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D68">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A68,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A68,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A68,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A68,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E68">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A68,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A68,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A68,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A68,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F68" s="5">
@@ -2156,22 +2158,22 @@
     </row>
     <row r="69">
       <c r="A69" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B69">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A69)+COUNTIFS('Post-GO'!A5:A61,$A69)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A69)+COUNTIFS('Post-GO'!A5:A62,$A69)</f>
         <v/>
       </c>
       <c r="C69">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A69,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A69,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A69,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A69,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D69">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A69,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A69,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A69,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A69,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E69">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A69,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A69,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A69,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A69,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F69" s="5">
@@ -2181,22 +2183,22 @@
     </row>
     <row r="70">
       <c r="A70" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B70">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A70)+COUNTIFS('Post-GO'!A5:A61,$A70)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A70)+COUNTIFS('Post-GO'!A5:A62,$A70)</f>
         <v/>
       </c>
       <c r="C70">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A70,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A70,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A70,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A70,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D70">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A70,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A70,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A70,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A70,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E70">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A70,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A70,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A70,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A70,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F70" s="5">
@@ -2205,25 +2207,23 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>8b</t>
-        </is>
+      <c r="A71" s="7" t="n">
+        <v>8</v>
       </c>
       <c r="B71">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A71)+COUNTIFS('Post-GO'!A5:A61,$A71)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A71)+COUNTIFS('Post-GO'!A5:A62,$A71)</f>
         <v/>
       </c>
       <c r="C71">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A71,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A71,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A71,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A71,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D71">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A71,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A71,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A71,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A71,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E71">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A71,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A71,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A71,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A71,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F71" s="5">
@@ -2232,23 +2232,25 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="n">
-        <v>9</v>
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>8b</t>
+        </is>
       </c>
       <c r="B72">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A72)+COUNTIFS('Post-GO'!A5:A61,$A72)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A72)+COUNTIFS('Post-GO'!A5:A62,$A72)</f>
         <v/>
       </c>
       <c r="C72">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A72,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A72,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A72,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A72,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D72">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A72,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A72,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A72,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A72,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E72">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A72,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A72,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A72,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A72,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F72" s="5">
@@ -2258,22 +2260,22 @@
     </row>
     <row r="73">
       <c r="A73" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B73">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A73)+COUNTIFS('Post-GO'!A5:A61,$A73)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A73)+COUNTIFS('Post-GO'!A5:A62,$A73)</f>
         <v/>
       </c>
       <c r="C73">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A73,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A73,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A73,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A73,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D73">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A73,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A73,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A73,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A73,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E73">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A73,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A73,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A73,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A73,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F73" s="5">
@@ -2283,22 +2285,22 @@
     </row>
     <row r="74">
       <c r="A74" s="7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B74">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A74)+COUNTIFS('Post-GO'!A5:A61,$A74)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A74)+COUNTIFS('Post-GO'!A5:A62,$A74)</f>
         <v/>
       </c>
       <c r="C74">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A74,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A74,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A74,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A74,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D74">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A74,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A74,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A74,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A74,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E74">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A74,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A74,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A74,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A74,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F74" s="5">
@@ -2308,26 +2310,51 @@
     </row>
     <row r="75">
       <c r="A75" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B75">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A75)+COUNTIFS('Post-GO'!A5:A61,$A75)</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A75)+COUNTIFS('Post-GO'!A5:A62,$A75)</f>
         <v/>
       </c>
       <c r="C75">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A75,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A61,$A75,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A75,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A75,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="D75">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A75,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A61,$A75,'Post-GO'!I5:I61,"In corso")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A75,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A75,'Post-GO'!I5:I62,"In corso")</f>
         <v/>
       </c>
       <c r="E75">
-        <f>COUNTIFS('Pre-GO'!A5:A26,$A75,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A61,$A75,'Post-GO'!I5:I61,"Da fare")</f>
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A75,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A75,'Post-GO'!I5:I62,"Da fare")</f>
         <v/>
       </c>
       <c r="F75" s="5">
         <f>IF(B75=0,0,C75/B75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B76">
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A76)+COUNTIFS('Post-GO'!A5:A62,$A76)</f>
+        <v/>
+      </c>
+      <c r="C76">
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A76,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!A5:A62,$A76,'Post-GO'!I5:I62,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="D76">
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A76,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!A5:A62,$A76,'Post-GO'!I5:I62,"In corso")</f>
+        <v/>
+      </c>
+      <c r="E76">
+        <f>COUNTIFS('Pre-GO'!A5:A26,$A76,'Pre-GO'!I5:I26,"Da fare")+COUNTIFS('Post-GO'!A5:A62,$A76,'Post-GO'!I5:I62,"Da fare")</f>
+        <v/>
+      </c>
+      <c r="F76" s="5">
+        <f>IF(B76=0,0,C76/B76)</f>
         <v/>
       </c>
     </row>
@@ -2344,7 +2371,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F21:F59">
+  <conditionalFormatting sqref="F21:F60">
     <cfRule type="dataBar" priority="2">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -2353,7 +2380,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F63:F75">
+  <conditionalFormatting sqref="F64:F76">
     <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -4499,7 +4526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V61"/>
+  <dimension ref="A1:V62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4540,11 +4567,11 @@
         </is>
       </c>
       <c r="B2" s="4">
-        <f>COUNTIF(I5:I61,"Fatto")/COUNTA(C5:C61)</f>
+        <f>COUNTIF(I5:I62,"Fatto")/COUNTA(C5:C62)</f>
         <v/>
       </c>
       <c r="C2">
-        <f>COUNTIF(I5:I61,"Fatto")&amp;" fatti / "&amp;COUNTA(C5:C61)&amp;" task · "&amp;COUNTIF(I5:I61,"In corso")&amp;" in corso · "&amp;COUNTIF(I5:I61,"Bloccato")&amp;" bloccati"</f>
+        <f>COUNTIF(I5:I62,"Fatto")&amp;" fatti / "&amp;COUNTA(C5:C62)&amp;" task · "&amp;COUNTIF(I5:I62,"In corso")&amp;" in corso · "&amp;COUNTIF(I5:I62,"Bloccato")&amp;" bloccati"</f>
         <v/>
       </c>
     </row>
@@ -6024,7 +6051,7 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Findings con severità/file/riga; non corregge</t>
+          <t>Findings con severità/file/riga **dall'enum di H-308** (Q-19); assegna la severità, **non decide cosa blocca**; non corregge; **può essere richiamato** sullo stesso task ai giri di rilavorazione (Q-20), dove verifica i *propri* findings e apre nuovi findings solo sul diff della correzione</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
@@ -7092,7 +7119,7 @@
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>`state.json`/`events.jsonl`, `STALE` dopo merge</t>
+          <t>`state.json`/`events.jsonl`, `STALE` dopo merge; lo stato include il **contatore dei giri di revisione** (Q-20), distinto da `maxAttempts`</t>
         </is>
       </c>
       <c r="H32" s="10" t="inlineStr">
@@ -7270,7 +7297,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Merge solo con tutti i gate; regressione fallisce prima del fix</t>
+          <t>Merge solo con tutti i gate; regressione fallisce prima del fix; **soglia di severità letta dalla policy** (Q-19)</t>
         </is>
       </c>
       <c r="H34" s="10" t="inlineStr">
@@ -7599,39 +7626,39 @@
     </row>
     <row r="38" ht="58" customHeight="1">
       <c r="A38" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B38" s="9" t="n">
         <v>56</v>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>H-612</t>
+          <t>H-716</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>PK-21</t>
+          <t>PK-19c</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>Valutazione rischi post-task (prodotto)</t>
+          <t>Ciclo di rilavorazione dei findings</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>**Fase 6, gruppo E.** T-611</t>
+          <t>**Fase 7.** Contatore **distinto** da R12 `maxAttempts`. T-716, E2E-REV-1</t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>`risk-assessor` al passaggio a VERIFIED (C28), `RISK-&lt;task&gt;.json` + `QUESTIONS.md`</t>
+          <t>`reviewer → developer → reviewer`, **max 2 correzioni**; al superamento `WAITING_SUPERVISOR`</t>
         </is>
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>H-308, H-701, H-706</t>
+          <t>H-607, H-711, H-308, H-706</t>
         </is>
       </c>
       <c r="I38" s="9" t="inlineStr">
@@ -7645,7 +7672,7 @@
       </c>
       <c r="K38" s="9" t="inlineStr">
         <is>
-          <t>NARO</t>
+          <t>SCIBETTA</t>
         </is>
       </c>
       <c r="L38" s="9" t="inlineStr"/>
@@ -7664,7 +7691,7 @@
       <c r="Q38" s="10" t="n"/>
       <c r="R38" s="10" t="inlineStr">
         <is>
-          <t>Dopo GO</t>
+          <t>Q-20. Dopo GO</t>
         </is>
       </c>
       <c r="S38" s="12" t="n">
@@ -7672,55 +7699,55 @@
       </c>
       <c r="T38" s="10" t="inlineStr">
         <is>
-          <t>T-611</t>
+          <t>T-716</t>
         </is>
       </c>
       <c r="U38" s="10" t="inlineStr">
         <is>
-          <t>H-308, H-701, H-706</t>
+          <t>H-308, H-607, H-706, H-711</t>
         </is>
       </c>
       <c r="V38" s="10" t="inlineStr">
         <is>
-          <t>agents/plugin/agents/risk-assessor.md, RISK-&lt;task&gt;.json</t>
+          <t>agents/plugin/ (ciclo reviewer-&gt;developer-&gt;reviewer, contatore dei giri), agents/policy/ (tetto dei giri)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="58" customHeight="1">
       <c r="A39" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39" s="9" t="n">
         <v>57</v>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>H-702</t>
+          <t>H-612</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>PK-22</t>
+          <t>PK-21</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>Installer `limet-agents.ps1/.sh`</t>
+          <t>Valutazione rischi post-task (prodotto)</t>
         </is>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>**Fase 7.** T-702</t>
+          <t>**Fase 6, gruppo E.** T-611</t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>`init|update` idempotente, plugin facoltativo</t>
+          <t>`risk-assessor` al passaggio a VERIFIED (C28), `RISK-&lt;task&gt;.json` + `QUESTIONS.md`</t>
         </is>
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t>gruppi A e C, H-407</t>
+          <t>H-308, H-701, H-706</t>
         </is>
       </c>
       <c r="I39" s="9" t="inlineStr">
@@ -7761,17 +7788,17 @@
       </c>
       <c r="T39" s="10" t="inlineStr">
         <is>
-          <t>T-702</t>
+          <t>T-611</t>
         </is>
       </c>
       <c r="U39" s="10" t="inlineStr">
         <is>
-          <t>H-407</t>
+          <t>H-308, H-701, H-706</t>
         </is>
       </c>
       <c r="V39" s="10" t="inlineStr">
         <is>
-          <t>scripts/limet-agents.ps1/.sh, limet/ (documentazione) [P]</t>
+          <t>agents/plugin/agents/risk-assessor.md, RISK-&lt;task&gt;.json</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7811,7 @@
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>H-712</t>
+          <t>H-702</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -7794,22 +7821,22 @@
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>Modifiche documentali a LIMET M.1–M.9</t>
+          <t>Installer `limet-agents.ps1/.sh`</t>
         </is>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>**Fase 7, gruppo F.** T-712</t>
+          <t>**Fase 7.** T-702</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>Ciclo LIMET IT/EN; re-index a cura dell'utente</t>
+          <t>`init|update` idempotente, plugin facoltativo</t>
         </is>
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>nessuna in IN; **[P]** dopo H-407 (ALA §7)</t>
+          <t>gruppi A e C, H-407</t>
         </is>
       </c>
       <c r="I40" s="9" t="inlineStr">
@@ -7850,7 +7877,7 @@
       </c>
       <c r="T40" s="10" t="inlineStr">
         <is>
-          <t>T-712</t>
+          <t>T-702</t>
         </is>
       </c>
       <c r="U40" s="10" t="inlineStr">
@@ -7866,39 +7893,39 @@
     </row>
     <row r="41" ht="58" customHeight="1">
       <c r="A41" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B41" s="9" t="n">
         <v>59</v>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>H-800</t>
+          <t>H-712</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>PK-23</t>
+          <t>PK-22</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>Analisi degli hook ECC</t>
+          <t>Modifiche documentali a LIMET M.1–M.9</t>
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8.** `docs/ecc-hooks-analysis.md`</t>
+          <t>**Fase 7, gruppo F.** T-712</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
-          <t>Decisione motivata per ognuno dei 27 hook</t>
+          <t>Ciclo LIMET IT/EN; re-index a cura dell'utente</t>
         </is>
       </c>
       <c r="H41" s="10" t="inlineStr">
         <is>
-          <t>H-401 [P]; anticipabile in Fase 2 (IN §5)</t>
+          <t>nessuna in IN; **[P]** dopo H-407 (ALA §7)</t>
         </is>
       </c>
       <c r="I41" s="9" t="inlineStr">
@@ -7912,7 +7939,7 @@
       </c>
       <c r="K41" s="9" t="inlineStr">
         <is>
-          <t>SCIBETTA</t>
+          <t>NARO</t>
         </is>
       </c>
       <c r="L41" s="9" t="inlineStr"/>
@@ -7931,7 +7958,7 @@
       <c r="Q41" s="10" t="n"/>
       <c r="R41" s="10" t="inlineStr">
         <is>
-          <t>Dopo GO (o anticipo)</t>
+          <t>Dopo GO</t>
         </is>
       </c>
       <c r="S41" s="12" t="n">
@@ -7939,17 +7966,17 @@
       </c>
       <c r="T41" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>T-712</t>
         </is>
       </c>
       <c r="U41" s="10" t="inlineStr">
         <is>
-          <t>H-401</t>
+          <t>H-407</t>
         </is>
       </c>
       <c r="V41" s="10" t="inlineStr">
         <is>
-          <t>docs/ecc-hooks-analysis.md</t>
+          <t>scripts/limet-agents.ps1/.sh, limet/ (documentazione) [P]</t>
         </is>
       </c>
     </row>
@@ -7962,7 +7989,7 @@
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>H-800b</t>
+          <t>H-800</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -7972,22 +7999,22 @@
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>Replica sicura hook utili</t>
+          <t>Analisi degli hook ECC</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8.** Verifica definita (audit A6): 5 criteri per hook — portabilità, nessuna rete, nessuna scrittura fuori workspace, log con hash, nessun file ECC in esecuzione. Nomi dei test dopo H-800 **[N]</t>
+          <t>**Fase 8.** `docs/ecc-hooks-analysis.md`</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>Hook HELIOS propri, mai codice ECC eseguito</t>
+          <t>Decisione motivata per ognuno dei 27 hook</t>
         </is>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>H-800</t>
+          <t>H-401 [P]; anticipabile in Fase 2 (IN §5)</t>
         </is>
       </c>
       <c r="I42" s="9" t="inlineStr">
@@ -8020,7 +8047,7 @@
       <c r="Q42" s="10" t="n"/>
       <c r="R42" s="10" t="inlineStr">
         <is>
-          <t>Dopo GO</t>
+          <t>Dopo GO (o anticipo)</t>
         </is>
       </c>
       <c r="S42" s="12" t="n">
@@ -8033,12 +8060,12 @@
       </c>
       <c r="U42" s="10" t="inlineStr">
         <is>
-          <t>H-800</t>
+          <t>H-401</t>
         </is>
       </c>
       <c r="V42" s="10" t="inlineStr">
         <is>
-          <t>docs/ecc-hooks-analysis.md, agents/policy/llm-registry.json, [N] wrapper AgentShield</t>
+          <t>docs/ecc-hooks-analysis.md</t>
         </is>
       </c>
     </row>
@@ -8051,7 +8078,7 @@
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>H-801</t>
+          <t>H-800b</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
@@ -8061,22 +8088,22 @@
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>Registro chiamate LLM (C05)</t>
+          <t>Replica sicura hook utili</t>
         </is>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8.** `agents/policy/llm-registry.json`</t>
+          <t>**Fase 8.** Verifica definita (audit A6): 5 criteri per hook — portabilità, nessuna rete, nessuna scrittura fuori workspace, log con hash, nessun file ECC in esecuzione. Nomi dei test dopo H-800 **[N]</t>
         </is>
       </c>
       <c r="G43" s="10" t="inlineStr">
         <is>
-          <t>Ogni chiamata LLM extra registrata</t>
+          <t>Hook HELIOS propri, mai codice ECC eseguito</t>
         </is>
       </c>
       <c r="H43" s="10" t="inlineStr">
         <is>
-          <t>H-401 [P]</t>
+          <t>H-800</t>
         </is>
       </c>
       <c r="I43" s="9" t="inlineStr">
@@ -8117,17 +8144,17 @@
       </c>
       <c r="T43" s="10" t="inlineStr">
         <is>
-          <t>T-801</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U43" s="10" t="inlineStr">
         <is>
-          <t>H-401</t>
+          <t>H-800</t>
         </is>
       </c>
       <c r="V43" s="10" t="inlineStr">
         <is>
-          <t>agents/policy/llm-registry.json</t>
+          <t>docs/ecc-hooks-analysis.md, agents/policy/llm-registry.json, [N] wrapper AgentShield</t>
         </is>
       </c>
     </row>
@@ -8140,7 +8167,7 @@
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>H-802</t>
+          <t>H-801</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -8150,17 +8177,17 @@
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>Wrapper AgentShield</t>
+          <t>Registro chiamate LLM (C05)</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8.** T-802. **[N]** licenze delle dipendenze (Q-10)</t>
+          <t>**Fase 8.** `agents/policy/llm-registry.json`</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>Pin, hash, SBOM, senza rete/`--opus`</t>
+          <t>Ogni chiamata LLM extra registrata</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
@@ -8206,7 +8233,7 @@
       </c>
       <c r="T44" s="10" t="inlineStr">
         <is>
-          <t>T-802</t>
+          <t>T-801</t>
         </is>
       </c>
       <c r="U44" s="10" t="inlineStr">
@@ -8216,7 +8243,7 @@
       </c>
       <c r="V44" s="10" t="inlineStr">
         <is>
-          <t>docs/ecc-hooks-analysis.md, agents/policy/llm-registry.json, [N] wrapper AgentShield</t>
+          <t>agents/policy/llm-registry.json</t>
         </is>
       </c>
     </row>
@@ -8229,32 +8256,32 @@
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>H-803</t>
+          <t>H-802</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>PK-24</t>
+          <t>PK-23</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>Setup KB `HLS_*`</t>
+          <t>Wrapper AgentShield</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8.** T-803 (Q9). Mai su collection esistenti</t>
+          <t>**Fase 8.** T-802. **[N]** licenze delle dipendenze (Q-10)</t>
         </is>
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>Crea `HLS_*` solo con autorizzazione esplicita del SUPERVISORE</t>
+          <t>Pin, hash, SBOM, senza rete/`--opus`</t>
         </is>
       </c>
       <c r="H45" s="10" t="inlineStr">
         <is>
-          <t>H-202, H-204 [P]</t>
+          <t>H-401 [P]</t>
         </is>
       </c>
       <c r="I45" s="9" t="inlineStr">
@@ -8295,17 +8322,17 @@
       </c>
       <c r="T45" s="10" t="inlineStr">
         <is>
-          <t>T-803</t>
+          <t>T-802</t>
         </is>
       </c>
       <c r="U45" s="10" t="inlineStr">
         <is>
-          <t>H-202, H-204</t>
+          <t>H-401</t>
         </is>
       </c>
       <c r="V45" s="10" t="inlineStr">
         <is>
-          <t>[N] script KB / MCP in sola lettura</t>
+          <t>docs/ecc-hooks-analysis.md, agents/policy/llm-registry.json, [N] wrapper AgentShield</t>
         </is>
       </c>
     </row>
@@ -8318,7 +8345,7 @@
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>H-804</t>
+          <t>H-803</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -8328,22 +8355,22 @@
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
-          <t>Accesso agenti alla KB</t>
+          <t>Setup KB `HLS_*`</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8.** T-804</t>
+          <t>**Fase 8.** T-803 (Q9). Mai su collection esistenti</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>Solo MCP/CLI in sola lettura, eventi registrati, degrado senza contesto</t>
+          <t>Crea `HLS_*` solo con autorizzazione esplicita del SUPERVISORE</t>
         </is>
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>H-803, H-611 [P]</t>
+          <t>H-202, H-204 [P]</t>
         </is>
       </c>
       <c r="I46" s="9" t="inlineStr">
@@ -8384,12 +8411,12 @@
       </c>
       <c r="T46" s="10" t="inlineStr">
         <is>
-          <t>T-804</t>
+          <t>T-803</t>
         </is>
       </c>
       <c r="U46" s="10" t="inlineStr">
         <is>
-          <t>H-611, H-803</t>
+          <t>H-202, H-204</t>
         </is>
       </c>
       <c r="V46" s="10" t="inlineStr">
@@ -8399,42 +8426,40 @@
       </c>
     </row>
     <row r="47" ht="58" customHeight="1">
-      <c r="A47" s="9" t="inlineStr">
-        <is>
-          <t>8b</t>
-        </is>
+      <c r="A47" s="9" t="n">
+        <v>8</v>
       </c>
       <c r="B47" s="9" t="n">
         <v>65</v>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>H-8b01</t>
+          <t>H-804</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>PK-25</t>
+          <t>PK-24</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>`api/` loopback e hardening</t>
+          <t>Accesso agenti alla KB</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** T-8b01…T-8b04</t>
+          <t>**Fase 8.** T-804</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>Token, Host/Origin, CSRF, CSP, limite body</t>
+          <t>Solo MCP/CLI in sola lettura, eventi registrati, degrado senza contesto</t>
         </is>
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>H-303, H-401 [P]</t>
+          <t>H-803, H-611 [P]</t>
         </is>
       </c>
       <c r="I47" s="9" t="inlineStr">
@@ -8475,17 +8500,17 @@
       </c>
       <c r="T47" s="10" t="inlineStr">
         <is>
-          <t>T-8b01, T-8b04</t>
+          <t>T-804</t>
         </is>
       </c>
       <c r="U47" s="10" t="inlineStr">
         <is>
-          <t>H-303, H-401</t>
+          <t>H-611, H-803</t>
         </is>
       </c>
       <c r="V47" s="10" t="inlineStr">
         <is>
-          <t>api/</t>
+          <t>[N] script KB / MCP in sola lettura</t>
         </is>
       </c>
     </row>
@@ -8500,7 +8525,7 @@
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>H-8b02</t>
+          <t>H-8b01</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -8510,22 +8535,22 @@
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>Read model derivato</t>
+          <t>`api/` loopback e hardening</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** T-8b05</t>
+          <t>**Fase 8b.** T-8b01…T-8b04</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>Cache rigenerabile, fonte unica (C27)</t>
+          <t>Token, Host/Origin, CSRF, CSP, limite body</t>
         </is>
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>H-8b01</t>
+          <t>H-303, H-401 [P]</t>
         </is>
       </c>
       <c r="I48" s="9" t="inlineStr">
@@ -8566,12 +8591,12 @@
       </c>
       <c r="T48" s="10" t="inlineStr">
         <is>
-          <t>T-8b05</t>
+          <t>T-8b01, T-8b04</t>
         </is>
       </c>
       <c r="U48" s="10" t="inlineStr">
         <is>
-          <t>H-8b01</t>
+          <t>H-303, H-401</t>
         </is>
       </c>
       <c r="V48" s="10" t="inlineStr">
@@ -8591,7 +8616,7 @@
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>H-8b05</t>
+          <t>H-8b02</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
@@ -8601,22 +8626,22 @@
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>Gate solo da sessione umana</t>
+          <t>Read model derivato</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** T-8b08 (C23–C24)</t>
+          <t>**Fase 8b.** T-8b05</t>
         </is>
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
-          <t>La UI non esegue build/test/git</t>
+          <t>Cache rigenerabile, fonte unica (C27)</t>
         </is>
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>H-8b01, H-403</t>
+          <t>H-8b01</t>
         </is>
       </c>
       <c r="I49" s="9" t="inlineStr">
@@ -8657,12 +8682,12 @@
       </c>
       <c r="T49" s="10" t="inlineStr">
         <is>
-          <t>T-8b08</t>
+          <t>T-8b05</t>
         </is>
       </c>
       <c r="U49" s="10" t="inlineStr">
         <is>
-          <t>H-403, H-8b01</t>
+          <t>H-8b01</t>
         </is>
       </c>
       <c r="V49" s="10" t="inlineStr">
@@ -8682,32 +8707,32 @@
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>H-8b03</t>
+          <t>H-8b05</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>PK-26</t>
+          <t>PK-25</t>
         </is>
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>`ui/` viste</t>
+          <t>Gate solo da sessione umana</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** T-8b06</t>
+          <t>**Fase 8b.** T-8b08 (C23–C24)</t>
         </is>
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
-          <t>Portfolio, LIMET, HELIOS, CEREBRO, Criticità</t>
+          <t>La UI non esegue build/test/git</t>
         </is>
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>H-8b02</t>
+          <t>H-8b01, H-403</t>
         </is>
       </c>
       <c r="I50" s="9" t="inlineStr">
@@ -8721,7 +8746,7 @@
       </c>
       <c r="K50" s="9" t="inlineStr">
         <is>
-          <t>NARO</t>
+          <t>SCIBETTA</t>
         </is>
       </c>
       <c r="L50" s="9" t="inlineStr"/>
@@ -8748,17 +8773,17 @@
       </c>
       <c r="T50" s="10" t="inlineStr">
         <is>
-          <t>T-8b06</t>
+          <t>T-8b08</t>
         </is>
       </c>
       <c r="U50" s="10" t="inlineStr">
         <is>
-          <t>H-8b02</t>
+          <t>H-403, H-8b01</t>
         </is>
       </c>
       <c r="V50" s="10" t="inlineStr">
         <is>
-          <t>ui/, [N] shim launcher :8799</t>
+          <t>api/</t>
         </is>
       </c>
     </row>
@@ -8773,7 +8798,7 @@
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>H-8b04</t>
+          <t>H-8b03</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
@@ -8783,22 +8808,22 @@
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>Vista Permessi agenti</t>
+          <t>`ui/` viste</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** T-405, T-8b07</t>
+          <t>**Fase 8b.** T-8b06</t>
         </is>
       </c>
       <c r="G51" s="10" t="inlineStr">
         <is>
-          <t>Conferma, motivazione, audit, rollback</t>
+          <t>Portfolio, LIMET, HELIOS, CEREBRO, Criticità</t>
         </is>
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>H-404, H-8b03</t>
+          <t>H-8b02</t>
         </is>
       </c>
       <c r="I51" s="9" t="inlineStr">
@@ -8839,12 +8864,12 @@
       </c>
       <c r="T51" s="10" t="inlineStr">
         <is>
-          <t>T-405, T-8b07</t>
+          <t>T-8b06</t>
         </is>
       </c>
       <c r="U51" s="10" t="inlineStr">
         <is>
-          <t>H-404, H-8b03</t>
+          <t>H-8b02</t>
         </is>
       </c>
       <c r="V51" s="10" t="inlineStr">
@@ -8864,7 +8889,7 @@
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>H-8b06</t>
+          <t>H-8b04</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -8874,22 +8899,22 @@
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>Grafica e accessibilità</t>
+          <t>Vista Permessi agenti</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** T-8b09</t>
+          <t>**Fase 8b.** T-405, T-8b07</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr">
         <is>
-          <t>SVG/Canvas, WCAG 2.1 AA, budget prestazioni (C26)</t>
+          <t>Conferma, motivazione, audit, rollback</t>
         </is>
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>H-8b03</t>
+          <t>H-404, H-8b03</t>
         </is>
       </c>
       <c r="I52" s="9" t="inlineStr">
@@ -8930,12 +8955,12 @@
       </c>
       <c r="T52" s="10" t="inlineStr">
         <is>
-          <t>T-8b09</t>
+          <t>T-405, T-8b07</t>
         </is>
       </c>
       <c r="U52" s="10" t="inlineStr">
         <is>
-          <t>H-8b03</t>
+          <t>H-404, H-8b03</t>
         </is>
       </c>
       <c r="V52" s="10" t="inlineStr">
@@ -8955,7 +8980,7 @@
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>H-8b07</t>
+          <t>H-8b06</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
@@ -8965,17 +8990,17 @@
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>Governance dipendenze npm</t>
+          <t>Grafica e accessibilità</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** T-8b10</t>
+          <t>**Fase 8b.** T-8b09</t>
         </is>
       </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
-          <t>Lockfile, licenze, audit, SBOM (C25)</t>
+          <t>SVG/Canvas, WCAG 2.1 AA, budget prestazioni (C26)</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
@@ -9021,7 +9046,7 @@
       </c>
       <c r="T53" s="10" t="inlineStr">
         <is>
-          <t>T-8b10</t>
+          <t>T-8b09</t>
         </is>
       </c>
       <c r="U53" s="10" t="inlineStr">
@@ -9046,7 +9071,7 @@
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>H-8b08</t>
+          <t>H-8b07</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -9056,22 +9081,22 @@
       </c>
       <c r="E54" s="10" t="inlineStr">
         <is>
-          <t>Sostituzione launcher :8799</t>
+          <t>Governance dipendenze npm</t>
         </is>
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** T-304</t>
+          <t>**Fase 8b.** T-8b10</t>
         </is>
       </c>
       <c r="G54" s="10" t="inlineStr">
         <is>
-          <t>Tramite shim</t>
+          <t>Lockfile, licenze, audit, SBOM (C25)</t>
         </is>
       </c>
       <c r="H54" s="10" t="inlineStr">
         <is>
-          <t>H-304, H-8b03</t>
+          <t>H-8b03</t>
         </is>
       </c>
       <c r="I54" s="9" t="inlineStr">
@@ -9112,12 +9137,12 @@
       </c>
       <c r="T54" s="10" t="inlineStr">
         <is>
-          <t>T-304</t>
+          <t>T-8b10</t>
         </is>
       </c>
       <c r="U54" s="10" t="inlineStr">
         <is>
-          <t>H-304, H-8b03</t>
+          <t>H-8b03</t>
         </is>
       </c>
       <c r="V54" s="10" t="inlineStr">
@@ -9137,32 +9162,32 @@
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>H-8b09</t>
+          <t>H-8b08</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>PK-26b</t>
+          <t>PK-26</t>
         </is>
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>Gate di configurazione all'avvio della dashboard</t>
+          <t>Sostituzione launcher :8799</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** Front-end del modulo H-309: stato `OK`/`INCOMPLETO`/`NON VALIDO`, dialog pre-compilata dall'autodiscovery, scrittura del file</t>
+          <t>**Fase 8b.** T-304</t>
         </is>
       </c>
       <c r="G55" s="10" t="inlineStr">
         <is>
-          <t>Nessuna operazione senza configurazione valida; dialog di prima configurazione</t>
+          <t>Tramite shim</t>
         </is>
       </c>
       <c r="H55" s="10" t="inlineStr">
         <is>
-          <t>H-309, H-8b01, H-8b03</t>
+          <t>H-304, H-8b03</t>
         </is>
       </c>
       <c r="I55" s="9" t="inlineStr">
@@ -9195,7 +9220,7 @@
       <c r="Q55" s="10" t="n"/>
       <c r="R55" s="10" t="inlineStr">
         <is>
-          <t>Dopo GO. Richiesta SUPERVISORE 2026-10-30</t>
+          <t>Dopo GO</t>
         </is>
       </c>
       <c r="S55" s="12" t="n">
@@ -9203,17 +9228,17 @@
       </c>
       <c r="T55" s="10" t="inlineStr">
         <is>
-          <t>T-8b11</t>
+          <t>T-304</t>
         </is>
       </c>
       <c r="U55" s="10" t="inlineStr">
         <is>
-          <t>H-309, H-8b01, H-8b03</t>
+          <t>H-304, H-8b03</t>
         </is>
       </c>
       <c r="V55" s="10" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>ui/, [N] shim launcher :8799</t>
         </is>
       </c>
     </row>
@@ -9228,32 +9253,32 @@
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>H-8b10</t>
+          <t>H-8b09</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>PK-26c</t>
+          <t>PK-26b</t>
         </is>
       </c>
       <c r="E56" s="10" t="inlineStr">
         <is>
-          <t>Avvio del run non presidiato dalla dashboard</t>
+          <t>Gate di configurazione all'avvio della dashboard</t>
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>**Fase 8b.** La UI non amplia i permessi (neutralità dei permessi, ADR 0003 §2). T-8b13, E2E-AUT-2</t>
+          <t>**Fase 8b.** Front-end del modulo H-309: stato `OK`/`INCOMPLETO`/`NON VALIDO`, dialog pre-compilata dall'autodiscovery, scrittura del file</t>
         </is>
       </c>
       <c r="G56" s="10" t="inlineStr">
         <is>
-          <t>Perimetro e limiti mostrati **prima** dell'avvio; avvio solo da sessione umana (C24); kill switch raggiungibile durante il run</t>
+          <t>Nessuna operazione senza configurazione valida; dialog di prima configurazione</t>
         </is>
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t>H-713, H-714, H-715, H-8b05</t>
+          <t>H-309, H-8b01, H-8b03</t>
         </is>
       </c>
       <c r="I56" s="9" t="inlineStr">
@@ -9286,7 +9311,7 @@
       <c r="Q56" s="10" t="n"/>
       <c r="R56" s="10" t="inlineStr">
         <is>
-          <t>Dopo GO. ADR 0003 §9</t>
+          <t>Dopo GO. Richiesta SUPERVISORE 2026-10-30</t>
         </is>
       </c>
       <c r="S56" s="12" t="n">
@@ -9294,55 +9319,57 @@
       </c>
       <c r="T56" s="10" t="inlineStr">
         <is>
-          <t>T-8b13, T-2</t>
+          <t>T-8b11</t>
         </is>
       </c>
       <c r="U56" s="10" t="inlineStr">
         <is>
-          <t>H-713, H-714, H-715, H-8b05</t>
+          <t>H-309, H-8b01, H-8b03</t>
         </is>
       </c>
       <c r="V56" s="10" t="inlineStr">
         <is>
-          <t>api/ (avvio run non presidiato), ui/ (pannello perimetro, limiti, kill switch)</t>
+          <t>/</t>
         </is>
       </c>
     </row>
     <row r="57" ht="58" customHeight="1">
-      <c r="A57" s="9" t="n">
-        <v>9</v>
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>8b</t>
+        </is>
       </c>
       <c r="B57" s="9" t="n">
         <v>75</v>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>H-901</t>
+          <t>H-8b10</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>PK-27</t>
+          <t>PK-26c</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>Scenari E2E ALA V1–V24</t>
+          <t>Avvio del run non presidiato dalla dashboard</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t>**Fase 9.** `E2E_VERIFICATION.md` (V1–V24)</t>
+          <t>**Fase 8b.** La UI non amplia i permessi (neutralità dei permessi, ADR 0003 §2). T-8b13, E2E-AUT-2</t>
         </is>
       </c>
       <c r="G57" s="10" t="inlineStr">
         <is>
-          <t>Catena completa su 3 OS, progetto pilota</t>
+          <t>Perimetro e limiti mostrati **prima** dell'avvio; avvio solo da sessione umana (C24); kill switch raggiungibile durante il run</t>
         </is>
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t>Fasi 5–8</t>
+          <t>H-713, H-714, H-715, H-8b05</t>
         </is>
       </c>
       <c r="I57" s="9" t="inlineStr">
@@ -9356,7 +9383,7 @@
       </c>
       <c r="K57" s="9" t="inlineStr">
         <is>
-          <t>SCIBETTA</t>
+          <t>NARO</t>
         </is>
       </c>
       <c r="L57" s="9" t="inlineStr"/>
@@ -9375,7 +9402,7 @@
       <c r="Q57" s="10" t="n"/>
       <c r="R57" s="10" t="inlineStr">
         <is>
-          <t>Dopo GO</t>
+          <t>Dopo GO. ADR 0003 §9</t>
         </is>
       </c>
       <c r="S57" s="12" t="n">
@@ -9383,17 +9410,17 @@
       </c>
       <c r="T57" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>T-8b13, T-2</t>
         </is>
       </c>
       <c r="U57" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>H-713, H-714, H-715, H-8b05</t>
         </is>
       </c>
       <c r="V57" s="10" t="inlineStr">
         <is>
-          <t>E2E_VERIFICATION.md</t>
+          <t>api/ (avvio run non presidiato), ui/ (pannello perimetro, limiti, kill switch)</t>
         </is>
       </c>
     </row>
@@ -9406,32 +9433,32 @@
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>H-902</t>
+          <t>H-901</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>PK-28</t>
+          <t>PK-27</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
         <is>
-          <t>README e troubleshooting plugin</t>
+          <t>Scenari E2E ALA V1–V24</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t>**Fase 9.** `agents/plugin/README.md`</t>
+          <t>**Fase 9.** `E2E_VERIFICATION.md` (V1–V24)</t>
         </is>
       </c>
       <c r="G58" s="10" t="inlineStr">
         <is>
-          <t>Installazione, configurazione, errori</t>
+          <t>Catena completa su 3 OS, progetto pilota</t>
         </is>
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>H-901 [P]</t>
+          <t>Fasi 5–8</t>
         </is>
       </c>
       <c r="I58" s="9" t="inlineStr">
@@ -9445,7 +9472,7 @@
       </c>
       <c r="K58" s="9" t="inlineStr">
         <is>
-          <t>NARO</t>
+          <t>SCIBETTA</t>
         </is>
       </c>
       <c r="L58" s="9" t="inlineStr"/>
@@ -9477,25 +9504,25 @@
       </c>
       <c r="U58" s="10" t="inlineStr">
         <is>
-          <t>H-901</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V58" s="10" t="inlineStr">
         <is>
-          <t>agents/plugin/README.md</t>
+          <t>E2E_VERIFICATION.md</t>
         </is>
       </c>
     </row>
     <row r="59" ht="58" customHeight="1">
       <c r="A59" s="9" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B59" s="9" t="n">
         <v>77</v>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>H-1101</t>
+          <t>H-902</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
@@ -9505,22 +9532,22 @@
       </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>Manuali, NOTICE, runbook</t>
+          <t>README e troubleshooting plugin</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>**Fase 11.** Revisione approvata</t>
+          <t>**Fase 9.** `agents/plugin/README.md`</t>
         </is>
       </c>
       <c r="G59" s="10" t="inlineStr">
         <is>
-          <t>Documentazione finale</t>
+          <t>Installazione, configurazione, errori</t>
         </is>
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t>H-901</t>
+          <t>H-901 [P]</t>
         </is>
       </c>
       <c r="I59" s="9" t="inlineStr">
@@ -9571,40 +9598,40 @@
       </c>
       <c r="V59" s="10" t="inlineStr">
         <is>
-          <t>agents/plugin/README.md, docs/ (manuali, NOTICE, runbook)</t>
+          <t>agents/plugin/README.md</t>
         </is>
       </c>
     </row>
     <row r="60" ht="58" customHeight="1">
       <c r="A60" s="9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B60" s="9" t="n">
         <v>78</v>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>H-1001</t>
+          <t>H-1101</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>PK-29</t>
+          <t>PK-28</t>
         </is>
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Manuali, NOTICE, runbook</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>**Fase 10.** Nessun T-xxx in IN §6 **[N]**: verifica = audit a 5 criteri osservabili (definita dall'audit A6), esito in `docs/audit-hardening.md`</t>
+          <t>**Fase 11.** Revisione approvata</t>
         </is>
       </c>
       <c r="G60" s="10" t="inlineStr">
         <is>
-          <t>Log immutabili, sandbox, SBOM, audit</t>
+          <t>Documentazione finale</t>
         </is>
       </c>
       <c r="H60" s="10" t="inlineStr">
@@ -9623,7 +9650,7 @@
       </c>
       <c r="K60" s="9" t="inlineStr">
         <is>
-          <t>SCIBETTA</t>
+          <t>NARO</t>
         </is>
       </c>
       <c r="L60" s="9" t="inlineStr"/>
@@ -9660,45 +9687,45 @@
       </c>
       <c r="V60" s="10" t="inlineStr">
         <is>
-          <t>docs/audit-hardening.md</t>
+          <t>agents/plugin/README.md, docs/ (manuali, NOTICE, runbook)</t>
         </is>
       </c>
     </row>
     <row r="61" ht="58" customHeight="1">
       <c r="A61" s="9" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B61" s="9" t="n">
         <v>79</v>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>H-1201</t>
+          <t>H-1001</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>PK-30</t>
+          <t>PK-29</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
         <is>
-          <t>Rollout sul pilota</t>
+          <t>Hardening</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>**Fase 12.** Parere legale **[N]**</t>
+          <t>**Fase 10.** Nessun T-xxx in IN §6 **[N]**: verifica = audit a 5 criteri osservabili (definita dall'audit A6), esito in `docs/audit-hardening.md`</t>
         </is>
       </c>
       <c r="G61" s="10" t="inlineStr">
         <is>
-          <t>Metriche, rollback, parere legale</t>
+          <t>Log immutabili, sandbox, SBOM, audit</t>
         </is>
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t>H-1001, H-1101</t>
+          <t>H-901</t>
         </is>
       </c>
       <c r="I61" s="9" t="inlineStr">
@@ -9712,7 +9739,7 @@
       </c>
       <c r="K61" s="9" t="inlineStr">
         <is>
-          <t>NARO</t>
+          <t>SCIBETTA</t>
         </is>
       </c>
       <c r="L61" s="9" t="inlineStr"/>
@@ -9744,21 +9771,110 @@
       </c>
       <c r="U61" s="10" t="inlineStr">
         <is>
+          <t>H-901</t>
+        </is>
+      </c>
+      <c r="V61" s="10" t="inlineStr">
+        <is>
+          <t>docs/audit-hardening.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="58" customHeight="1">
+      <c r="A62" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B62" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>H-1201</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>PK-30</t>
+        </is>
+      </c>
+      <c r="E62" s="10" t="inlineStr">
+        <is>
+          <t>Rollout sul pilota</t>
+        </is>
+      </c>
+      <c r="F62" s="10" t="inlineStr">
+        <is>
+          <t>**Fase 12.** Parere legale **[N]**</t>
+        </is>
+      </c>
+      <c r="G62" s="10" t="inlineStr">
+        <is>
+          <t>Metriche, rollback, parere legale</t>
+        </is>
+      </c>
+      <c r="H62" s="10" t="inlineStr">
+        <is>
           <t>H-1001, H-1101</t>
         </is>
       </c>
-      <c r="V61" s="10" t="inlineStr">
+      <c r="I62" s="9" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="J62" s="9">
+        <f>IF(I62="Fatto","✔ Sì","✘ No")</f>
+        <v/>
+      </c>
+      <c r="K62" s="9" t="inlineStr">
+        <is>
+          <t>NARO</t>
+        </is>
+      </c>
+      <c r="L62" s="9" t="inlineStr"/>
+      <c r="M62" s="10" t="inlineStr"/>
+      <c r="N62" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O62" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P62" s="10" t="n"/>
+      <c r="Q62" s="10" t="n"/>
+      <c r="R62" s="10" t="inlineStr">
+        <is>
+          <t>Dopo GO</t>
+        </is>
+      </c>
+      <c r="S62" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T62" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U62" s="10" t="inlineStr">
+        <is>
+          <t>H-1001, H-1101</t>
+        </is>
+      </c>
+      <c r="V62" s="10" t="inlineStr">
         <is>
           <t>docs/ (metriche, rollback)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:V61"/>
+  <autoFilter ref="A4:V62"/>
   <mergeCells count="1">
     <mergeCell ref="A1:V1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:S61">
+  <conditionalFormatting sqref="A5:S62">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND($S5=1,$I5&lt;&gt;"Fatto")</formula>
     </cfRule>
@@ -9766,7 +9882,7 @@
       <formula>$I5="Fatto"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I61">
+  <conditionalFormatting sqref="I5:I62">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"Fatto"</formula>
     </cfRule>
@@ -9783,7 +9899,7 @@
       <formula>"Da fare"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K61">
+  <conditionalFormatting sqref="K5:K62">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
       <formula>"NARO"</formula>
     </cfRule>
@@ -9794,7 +9910,7 @@
       <formula>"SUPERVISORE"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S5:S61">
+  <conditionalFormatting sqref="S5:S62">
     <cfRule type="dataBar" priority="11">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -9804,19 +9920,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="I5:I61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I5:I62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da fare,In corso,In review,Fatto,Bloccato"</formula1>
     </dataValidation>
-    <dataValidation sqref="K5:K61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NARO,SCIBETTA,SUPERVISORE,Da assegnare"</formula1>
     </dataValidation>
-    <dataValidation sqref="L5:L61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L5:L62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"S,M,L"</formula1>
     </dataValidation>
-    <dataValidation sqref="N5:N61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N5:N62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sì,No,—"</formula1>
     </dataValidation>
-    <dataValidation sqref="S5:S61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
+    <dataValidation sqref="S5:S62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -9832,7 +9948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9959,15 +10075,15 @@
         </is>
       </c>
       <c r="E5" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A5)+COUNTIF('Post-GO'!D5:D61,A5)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A5)+COUNTIF('Post-GO'!D5:D62,A5)</f>
         <v/>
       </c>
       <c r="F5" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A5,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A5,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A5,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A5,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G5" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A5,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A5,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F5=E5,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A5,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A5,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A5,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A5,'Post-GO'!I5:I61,"In review")+F5&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A5,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A5,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F5=E5,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A5,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A5,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A5,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A5,'Post-GO'!I5:I62,"In review")+F5&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H5" s="9" t="inlineStr">
@@ -10028,15 +10144,15 @@
         </is>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A6)+COUNTIF('Post-GO'!D5:D61,A6)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A6)+COUNTIF('Post-GO'!D5:D62,A6)</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A6,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A6,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A6,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A6,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G6" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A6,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A6,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F6=E6,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A6,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A6,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A6,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A6,'Post-GO'!I5:I61,"In review")+F6&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A6,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A6,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F6=E6,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A6,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A6,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A6,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A6,'Post-GO'!I5:I62,"In review")+F6&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -10097,15 +10213,15 @@
         </is>
       </c>
       <c r="E7" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A7)+COUNTIF('Post-GO'!D5:D61,A7)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A7)+COUNTIF('Post-GO'!D5:D62,A7)</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A7,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A7,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A7,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A7,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A7,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A7,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F7=E7,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A7,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A7,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A7,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A7,'Post-GO'!I5:I61,"In review")+F7&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A7,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A7,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F7=E7,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A7,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A7,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A7,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A7,'Post-GO'!I5:I62,"In review")+F7&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H7" s="9" t="inlineStr">
@@ -10166,15 +10282,15 @@
         </is>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A8)+COUNTIF('Post-GO'!D5:D61,A8)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A8)+COUNTIF('Post-GO'!D5:D62,A8)</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A8,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A8,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A8,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A8,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A8,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A8,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F8=E8,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A8,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A8,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A8,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A8,'Post-GO'!I5:I61,"In review")+F8&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A8,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A8,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F8=E8,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A8,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A8,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A8,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A8,'Post-GO'!I5:I62,"In review")+F8&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H8" s="9" t="inlineStr">
@@ -10235,15 +10351,15 @@
         </is>
       </c>
       <c r="E9" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A9)+COUNTIF('Post-GO'!D5:D61,A9)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A9)+COUNTIF('Post-GO'!D5:D62,A9)</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A9,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A9,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A9,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A9,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A9,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A9,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F9=E9,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A9,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A9,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A9,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A9,'Post-GO'!I5:I61,"In review")+F9&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A9,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A9,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F9=E9,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A9,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A9,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A9,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A9,'Post-GO'!I5:I62,"In review")+F9&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H9" s="9" t="inlineStr">
@@ -10304,15 +10420,15 @@
         </is>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A10)+COUNTIF('Post-GO'!D5:D61,A10)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A10)+COUNTIF('Post-GO'!D5:D62,A10)</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A10,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A10,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A10,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A10,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G10" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A10,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A10,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F10=E10,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A10,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A10,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A10,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A10,'Post-GO'!I5:I61,"In review")+F10&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A10,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A10,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F10=E10,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A10,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A10,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A10,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A10,'Post-GO'!I5:I62,"In review")+F10&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H10" s="9" t="inlineStr">
@@ -10373,15 +10489,15 @@
         </is>
       </c>
       <c r="E11" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A11)+COUNTIF('Post-GO'!D5:D61,A11)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A11)+COUNTIF('Post-GO'!D5:D62,A11)</f>
         <v/>
       </c>
       <c r="F11" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A11,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A11,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A11,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A11,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G11" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A11,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A11,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F11=E11,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A11,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A11,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A11,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A11,'Post-GO'!I5:I61,"In review")+F11&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A11,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A11,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F11=E11,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A11,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A11,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A11,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A11,'Post-GO'!I5:I62,"In review")+F11&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H11" s="9" t="inlineStr">
@@ -10442,15 +10558,15 @@
         </is>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A12)+COUNTIF('Post-GO'!D5:D61,A12)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A12)+COUNTIF('Post-GO'!D5:D62,A12)</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A12,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A12,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A12,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A12,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G12" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A12,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A12,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F12=E12,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A12,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A12,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A12,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A12,'Post-GO'!I5:I61,"In review")+F12&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A12,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A12,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F12=E12,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A12,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A12,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A12,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A12,'Post-GO'!I5:I62,"In review")+F12&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H12" s="9" t="inlineStr">
@@ -10511,15 +10627,15 @@
         </is>
       </c>
       <c r="E13" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A13)+COUNTIF('Post-GO'!D5:D61,A13)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A13)+COUNTIF('Post-GO'!D5:D62,A13)</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A13,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A13,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A13,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A13,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G13" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A13,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A13,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F13=E13,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A13,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A13,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A13,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A13,'Post-GO'!I5:I61,"In review")+F13&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A13,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A13,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F13=E13,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A13,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A13,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A13,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A13,'Post-GO'!I5:I62,"In review")+F13&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H13" s="9" t="inlineStr">
@@ -10580,15 +10696,15 @@
         </is>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A14)+COUNTIF('Post-GO'!D5:D61,A14)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A14)+COUNTIF('Post-GO'!D5:D62,A14)</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A14,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A14,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A14,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A14,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A14,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A14,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F14=E14,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A14,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A14,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A14,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A14,'Post-GO'!I5:I61,"In review")+F14&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A14,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A14,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F14=E14,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A14,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A14,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A14,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A14,'Post-GO'!I5:I62,"In review")+F14&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H14" s="9" t="inlineStr">
@@ -10649,15 +10765,15 @@
         </is>
       </c>
       <c r="E15" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A15)+COUNTIF('Post-GO'!D5:D61,A15)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A15)+COUNTIF('Post-GO'!D5:D62,A15)</f>
         <v/>
       </c>
       <c r="F15" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A15,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A15,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A15,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A15,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G15" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A15,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A15,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F15=E15,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A15,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A15,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A15,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A15,'Post-GO'!I5:I61,"In review")+F15&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A15,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A15,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F15=E15,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A15,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A15,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A15,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A15,'Post-GO'!I5:I62,"In review")+F15&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H15" s="9" t="inlineStr">
@@ -10718,15 +10834,15 @@
         </is>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A16)+COUNTIF('Post-GO'!D5:D61,A16)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A16)+COUNTIF('Post-GO'!D5:D62,A16)</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A16,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A16,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A16,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A16,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G16" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A16,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A16,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F16=E16,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A16,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A16,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A16,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A16,'Post-GO'!I5:I61,"In review")+F16&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A16,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A16,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F16=E16,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A16,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A16,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A16,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A16,'Post-GO'!I5:I62,"In review")+F16&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H16" s="9" t="inlineStr">
@@ -10787,15 +10903,15 @@
         </is>
       </c>
       <c r="E17" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A17)+COUNTIF('Post-GO'!D5:D61,A17)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A17)+COUNTIF('Post-GO'!D5:D62,A17)</f>
         <v/>
       </c>
       <c r="F17" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A17,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A17,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A17,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A17,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G17" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A17,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A17,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F17=E17,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A17,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A17,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A17,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A17,'Post-GO'!I5:I61,"In review")+F17&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A17,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A17,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F17=E17,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A17,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A17,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A17,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A17,'Post-GO'!I5:I62,"In review")+F17&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H17" s="9" t="inlineStr">
@@ -10856,15 +10972,15 @@
         </is>
       </c>
       <c r="E18" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A18)+COUNTIF('Post-GO'!D5:D61,A18)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A18)+COUNTIF('Post-GO'!D5:D62,A18)</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A18,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A18,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A18,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A18,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A18,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A18,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F18=E18,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A18,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A18,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A18,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A18,'Post-GO'!I5:I61,"In review")+F18&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A18,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A18,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F18=E18,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A18,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A18,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A18,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A18,'Post-GO'!I5:I62,"In review")+F18&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H18" s="9" t="inlineStr">
@@ -10925,15 +11041,15 @@
         </is>
       </c>
       <c r="E19" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A19)+COUNTIF('Post-GO'!D5:D61,A19)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A19)+COUNTIF('Post-GO'!D5:D62,A19)</f>
         <v/>
       </c>
       <c r="F19" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A19,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A19,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A19,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A19,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G19" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A19,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A19,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F19=E19,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A19,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A19,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A19,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A19,'Post-GO'!I5:I61,"In review")+F19&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A19,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A19,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F19=E19,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A19,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A19,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A19,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A19,'Post-GO'!I5:I62,"In review")+F19&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H19" s="9" t="inlineStr">
@@ -10994,15 +11110,15 @@
         </is>
       </c>
       <c r="E20" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A20)+COUNTIF('Post-GO'!D5:D61,A20)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A20)+COUNTIF('Post-GO'!D5:D62,A20)</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A20,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A20,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A20,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A20,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G20" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A20,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A20,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F20=E20,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A20,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A20,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A20,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A20,'Post-GO'!I5:I61,"In review")+F20&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A20,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A20,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F20=E20,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A20,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A20,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A20,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A20,'Post-GO'!I5:I62,"In review")+F20&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H20" s="9" t="inlineStr">
@@ -11063,15 +11179,15 @@
         </is>
       </c>
       <c r="E21" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A21)+COUNTIF('Post-GO'!D5:D61,A21)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A21)+COUNTIF('Post-GO'!D5:D62,A21)</f>
         <v/>
       </c>
       <c r="F21" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A21,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A21,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A21,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A21,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G21" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A21,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A21,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F21=E21,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A21,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A21,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A21,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A21,'Post-GO'!I5:I61,"In review")+F21&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A21,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A21,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F21=E21,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A21,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A21,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A21,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A21,'Post-GO'!I5:I62,"In review")+F21&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H21" s="9" t="inlineStr">
@@ -11132,15 +11248,15 @@
         </is>
       </c>
       <c r="E22" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A22)+COUNTIF('Post-GO'!D5:D61,A22)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A22)+COUNTIF('Post-GO'!D5:D62,A22)</f>
         <v/>
       </c>
       <c r="F22" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A22,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A22,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A22,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A22,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G22" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A22,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A22,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F22=E22,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A22,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A22,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A22,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A22,'Post-GO'!I5:I61,"In review")+F22&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A22,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A22,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F22=E22,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A22,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A22,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A22,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A22,'Post-GO'!I5:I62,"In review")+F22&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -11201,15 +11317,15 @@
         </is>
       </c>
       <c r="E23" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A23)+COUNTIF('Post-GO'!D5:D61,A23)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A23)+COUNTIF('Post-GO'!D5:D62,A23)</f>
         <v/>
       </c>
       <c r="F23" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A23,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A23,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A23,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A23,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G23" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A23,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A23,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F23=E23,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A23,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A23,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A23,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A23,'Post-GO'!I5:I61,"In review")+F23&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A23,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A23,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F23=E23,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A23,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A23,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A23,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A23,'Post-GO'!I5:I62,"In review")+F23&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H23" s="9" t="inlineStr">
@@ -11270,15 +11386,15 @@
         </is>
       </c>
       <c r="E24" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A24)+COUNTIF('Post-GO'!D5:D61,A24)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A24)+COUNTIF('Post-GO'!D5:D62,A24)</f>
         <v/>
       </c>
       <c r="F24" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A24,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A24,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A24,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A24,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G24" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A24,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A24,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F24=E24,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A24,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A24,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A24,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A24,'Post-GO'!I5:I61,"In review")+F24&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A24,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A24,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F24=E24,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A24,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A24,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A24,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A24,'Post-GO'!I5:I62,"In review")+F24&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H24" s="9" t="inlineStr">
@@ -11339,15 +11455,15 @@
         </is>
       </c>
       <c r="E25" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A25)+COUNTIF('Post-GO'!D5:D61,A25)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A25)+COUNTIF('Post-GO'!D5:D62,A25)</f>
         <v/>
       </c>
       <c r="F25" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A25,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A25,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A25,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A25,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G25" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A25,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A25,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F25=E25,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A25,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A25,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A25,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A25,'Post-GO'!I5:I61,"In review")+F25&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A25,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A25,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F25=E25,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A25,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A25,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A25,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A25,'Post-GO'!I5:I62,"In review")+F25&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H25" s="9" t="inlineStr">
@@ -11408,15 +11524,15 @@
         </is>
       </c>
       <c r="E26" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A26)+COUNTIF('Post-GO'!D5:D61,A26)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A26)+COUNTIF('Post-GO'!D5:D62,A26)</f>
         <v/>
       </c>
       <c r="F26" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A26,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A26,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A26,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A26,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G26" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A26,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A26,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F26=E26,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A26,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A26,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A26,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A26,'Post-GO'!I5:I61,"In review")+F26&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A26,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A26,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F26=E26,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A26,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A26,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A26,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A26,'Post-GO'!I5:I62,"In review")+F26&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H26" s="9" t="inlineStr">
@@ -11477,15 +11593,15 @@
         </is>
       </c>
       <c r="E27" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A27)+COUNTIF('Post-GO'!D5:D61,A27)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A27)+COUNTIF('Post-GO'!D5:D62,A27)</f>
         <v/>
       </c>
       <c r="F27" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A27,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A27,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A27,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A27,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G27" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A27,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A27,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F27=E27,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A27,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A27,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A27,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A27,'Post-GO'!I5:I61,"In review")+F27&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A27,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A27,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F27=E27,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A27,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A27,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A27,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A27,'Post-GO'!I5:I62,"In review")+F27&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H27" s="9" t="inlineStr">
@@ -11546,15 +11662,15 @@
         </is>
       </c>
       <c r="E28" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A28)+COUNTIF('Post-GO'!D5:D61,A28)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A28)+COUNTIF('Post-GO'!D5:D62,A28)</f>
         <v/>
       </c>
       <c r="F28" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A28,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A28,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A28,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A28,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G28" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A28,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A28,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F28=E28,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A28,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A28,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A28,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A28,'Post-GO'!I5:I61,"In review")+F28&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A28,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A28,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F28=E28,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A28,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A28,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A28,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A28,'Post-GO'!I5:I62,"In review")+F28&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H28" s="9" t="inlineStr">
@@ -11615,15 +11731,15 @@
         </is>
       </c>
       <c r="E29" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A29)+COUNTIF('Post-GO'!D5:D61,A29)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A29)+COUNTIF('Post-GO'!D5:D62,A29)</f>
         <v/>
       </c>
       <c r="F29" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A29,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A29,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A29,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A29,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G29" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A29,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A29,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F29=E29,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A29,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A29,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A29,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A29,'Post-GO'!I5:I61,"In review")+F29&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A29,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A29,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F29=E29,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A29,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A29,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A29,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A29,'Post-GO'!I5:I62,"In review")+F29&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H29" s="9" t="inlineStr">
@@ -11684,15 +11800,15 @@
         </is>
       </c>
       <c r="E30" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A30)+COUNTIF('Post-GO'!D5:D61,A30)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A30)+COUNTIF('Post-GO'!D5:D62,A30)</f>
         <v/>
       </c>
       <c r="F30" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A30,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A30,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A30,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A30,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G30" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A30,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A30,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F30=E30,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A30,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A30,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A30,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A30,'Post-GO'!I5:I61,"In review")+F30&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A30,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A30,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F30=E30,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A30,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A30,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A30,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A30,'Post-GO'!I5:I62,"In review")+F30&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H30" s="9" t="inlineStr">
@@ -11753,15 +11869,15 @@
         </is>
       </c>
       <c r="E31" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A31)+COUNTIF('Post-GO'!D5:D61,A31)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A31)+COUNTIF('Post-GO'!D5:D62,A31)</f>
         <v/>
       </c>
       <c r="F31" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A31,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A31,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A31,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A31,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G31" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A31,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A31,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F31=E31,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A31,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A31,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A31,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A31,'Post-GO'!I5:I61,"In review")+F31&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A31,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A31,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F31=E31,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A31,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A31,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A31,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A31,'Post-GO'!I5:I62,"In review")+F31&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H31" s="9" t="inlineStr">
@@ -11803,103 +11919,103 @@
     <row r="32" ht="62" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>PK-21</t>
+          <t>PK-19c</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Onda 6 (dopo GO)</t>
+          <t>Onda 5+ (dopo GO)</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Valutazione rischi di prodotto (C28)</t>
+          <t>Ciclo di rilavorazione dei findings di code review</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>H-612</t>
+          <t>H-716</t>
         </is>
       </c>
       <c r="E32" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A32)+COUNTIF('Post-GO'!D5:D61,A32)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A32)+COUNTIF('Post-GO'!D5:D62,A32)</f>
         <v/>
       </c>
       <c r="F32" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A32,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A32,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A32,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A32,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G32" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A32,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A32,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F32=E32,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A32,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A32,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A32,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A32,'Post-GO'!I5:I61,"In review")+F32&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A32,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A32,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F32=E32,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A32,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A32,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A32,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A32,'Post-GO'!I5:I62,"In review")+F32&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>NARO</t>
+          <t>SCIBETTA</t>
         </is>
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
-          <t>N11</t>
+          <t>S9c</t>
         </is>
       </c>
       <c r="J32" s="10" t="inlineStr">
         <is>
-          <t>T-611</t>
+          <t>T-716</t>
         </is>
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>agents/plugin/agents/risk-assessor.md, RISK-&lt;task&gt;.json</t>
+          <t>agents/plugin/ (ciclo reviewer-&gt;developer-&gt;reviewer, contatore dei giri), agents/policy/ (tetto dei giri)</t>
         </is>
       </c>
       <c r="L32" s="10" t="inlineStr">
         <is>
-          <t>PK-19 (H-701), PK-20 (H-706), H-308</t>
+          <t>PK-18 (H-607), PK-19 (H-701), PK-20 (H-706, H-711)</t>
         </is>
       </c>
       <c r="M32" s="10" t="inlineStr">
         <is>
-          <t>PK-23, PK-24, PK-25</t>
+          <t>PK-20</t>
         </is>
       </c>
       <c r="N32" s="10" t="inlineStr">
         <is>
-          <t>risk-assessor ≠ developer, sola lettura.</t>
+          <t>Q-20. Max 2 correzioni, poi WAITING_SUPERVISOR. Contatore dei giri DISTINTO da R12 maxAttempts. Stessi file di PK-19 (limet-change.js): stessa persona. Contatto con PK-20 sul contratto di stato. Verifica: T-716, E2E-REV-1.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="62" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>PK-22</t>
+          <t>PK-21</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Onda 5 (dopo GO)</t>
+          <t>Onda 6 (dopo GO)</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Installer e modifiche documentali a LIMET</t>
+          <t>Valutazione rischi di prodotto (C28)</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>H-702, H-712</t>
+          <t>H-612</t>
         </is>
       </c>
       <c r="E33" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A33)+COUNTIF('Post-GO'!D5:D61,A33)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A33)+COUNTIF('Post-GO'!D5:D62,A33)</f>
         <v/>
       </c>
       <c r="F33" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A33,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A33,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A33,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A33,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G33" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A33,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A33,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F33=E33,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A33,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A33,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A33,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A33,'Post-GO'!I5:I61,"In review")+F33&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A33,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A33,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F33=E33,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A33,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A33,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A33,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A33,'Post-GO'!I5:I62,"In review")+F33&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H33" s="9" t="inlineStr">
@@ -11909,135 +12025,135 @@
       </c>
       <c r="I33" s="9" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>N11</t>
         </is>
       </c>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>T-702, T-712</t>
+          <t>T-611</t>
         </is>
       </c>
       <c r="K33" s="10" t="inlineStr">
         <is>
-          <t>scripts/limet-agents.ps1/.sh, limet/ (documentazione) [P]</t>
+          <t>agents/plugin/agents/risk-assessor.md, RISK-&lt;task&gt;.json</t>
         </is>
       </c>
       <c r="L33" s="10" t="inlineStr">
         <is>
-          <t>H-407; H-712 dopo H-407 (ALA §7)</t>
+          <t>PK-19 (H-701), PK-20 (H-706), H-308</t>
         </is>
       </c>
       <c r="M33" s="10" t="inlineStr">
         <is>
-          <t>PK-19</t>
+          <t>PK-23, PK-24, PK-25</t>
         </is>
       </c>
       <c r="N33" s="10" t="inlineStr">
         <is>
-          <t>Ciclo LIMET IT/EN; re-index a cura del SUPERVISORE.</t>
+          <t>risk-assessor ≠ developer, sola lettura.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="62" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>PK-23</t>
+          <t>PK-22</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Onda 3+ (dopo GO)</t>
+          <t>Onda 5 (dopo GO)</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Hook ECC e registro chiamate LLM</t>
+          <t>Installer e modifiche documentali a LIMET</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>H-800, H-800b, H-801, H-802</t>
+          <t>H-702, H-712</t>
         </is>
       </c>
       <c r="E34" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A34)+COUNTIF('Post-GO'!D5:D61,A34)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A34)+COUNTIF('Post-GO'!D5:D62,A34)</f>
         <v/>
       </c>
       <c r="F34" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A34,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A34,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A34,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A34,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G34" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A34,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A34,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F34=E34,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A34,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A34,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A34,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A34,'Post-GO'!I5:I61,"In review")+F34&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A34,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A34,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F34=E34,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A34,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A34,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A34,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A34,'Post-GO'!I5:I62,"In review")+F34&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>SCIBETTA</t>
+          <t>NARO</t>
         </is>
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>N12</t>
         </is>
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
-          <t>T-801, T-802</t>
+          <t>T-702, T-712</t>
         </is>
       </c>
       <c r="K34" s="10" t="inlineStr">
         <is>
-          <t>docs/ecc-hooks-analysis.md, agents/policy/llm-registry.json, [N] wrapper AgentShield</t>
+          <t>scripts/limet-agents.ps1/.sh, limet/ (documentazione) [P]</t>
         </is>
       </c>
       <c r="L34" s="10" t="inlineStr">
         <is>
-          <t>GO; PK-08</t>
+          <t>H-407; H-712 dopo H-407 (ALA §7)</t>
         </is>
       </c>
       <c r="M34" s="10" t="inlineStr">
         <is>
-          <t>PK-14…PK-22</t>
+          <t>PK-19</t>
         </is>
       </c>
       <c r="N34" s="10" t="inlineStr">
         <is>
-          <t>H-800 anticipabile in Fase 2 (IN §5). [N] Q-10 licenze AgentShield.</t>
+          <t>Ciclo LIMET IT/EN; re-index a cura del SUPERVISORE.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="62" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>PK-24</t>
+          <t>PK-23</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Onda 6 (dopo GO)</t>
+          <t>Onda 3+ (dopo GO)</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Knowledge base HLS_* e accesso agenti</t>
+          <t>Hook ECC e registro chiamate LLM</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>H-803, H-804</t>
+          <t>H-800, H-800b, H-801, H-802</t>
         </is>
       </c>
       <c r="E35" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A35)+COUNTIF('Post-GO'!D5:D61,A35)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A35)+COUNTIF('Post-GO'!D5:D62,A35)</f>
         <v/>
       </c>
       <c r="F35" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A35,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A35,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A35,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A35,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G35" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A35,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A35,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F35=E35,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A35,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A35,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A35,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A35,'Post-GO'!I5:I61,"In review")+F35&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A35,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A35,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F35=E35,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A35,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A35,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A35,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A35,'Post-GO'!I5:I62,"In review")+F35&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H35" s="9" t="inlineStr">
@@ -12047,66 +12163,66 @@
       </c>
       <c r="I35" s="9" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>T-803, T-804</t>
+          <t>T-801, T-802</t>
         </is>
       </c>
       <c r="K35" s="10" t="inlineStr">
         <is>
-          <t>[N] script KB / MCP in sola lettura</t>
+          <t>docs/ecc-hooks-analysis.md, agents/policy/llm-registry.json, [N] wrapper AgentShield</t>
         </is>
       </c>
       <c r="L35" s="10" t="inlineStr">
         <is>
-          <t>PK-03, PK-15</t>
+          <t>GO; PK-08</t>
         </is>
       </c>
       <c r="M35" s="10" t="inlineStr">
         <is>
-          <t>PK-21</t>
+          <t>PK-14…PK-22</t>
         </is>
       </c>
       <c r="N35" s="10" t="inlineStr">
         <is>
-          <t>HLS_* creata solo con autorizzazione esplicita (Q9); mai su collection esistenti.</t>
+          <t>H-800 anticipabile in Fase 2 (IN §5). [N] Q-10 licenze AgentShield.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="62" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>PK-25</t>
+          <t>PK-24</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Onda 3+ (dopo GO)</t>
+          <t>Onda 6 (dopo GO)</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>API loopback e read model</t>
+          <t>Knowledge base HLS_* e accesso agenti</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>H-8b01, H-8b02, H-8b05</t>
+          <t>H-803, H-804</t>
         </is>
       </c>
       <c r="E36" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A36)+COUNTIF('Post-GO'!D5:D61,A36)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A36)+COUNTIF('Post-GO'!D5:D62,A36)</f>
         <v/>
       </c>
       <c r="F36" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A36,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A36,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A36,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A36,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G36" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A36,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A36,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F36=E36,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A36,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A36,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A36,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A36,'Post-GO'!I5:I61,"In review")+F36&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A36,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A36,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F36=E36,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A36,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A36,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A36,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A36,'Post-GO'!I5:I62,"In review")+F36&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H36" s="9" t="inlineStr">
@@ -12116,108 +12232,108 @@
       </c>
       <c r="I36" s="9" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>T-8b01, T-8b04, T-8b05, T-8b08</t>
+          <t>T-803, T-804</t>
         </is>
       </c>
       <c r="K36" s="10" t="inlineStr">
         <is>
-          <t>api/</t>
+          <t>[N] script KB / MCP in sola lettura</t>
         </is>
       </c>
       <c r="L36" s="10" t="inlineStr">
         <is>
-          <t>GO; PK-06, PK-08</t>
+          <t>PK-03, PK-15</t>
         </is>
       </c>
       <c r="M36" s="10" t="inlineStr">
         <is>
-          <t>PK-26 (dopo contratto API)</t>
+          <t>PK-21</t>
         </is>
       </c>
       <c r="N36" s="10" t="inlineStr">
         <is>
-          <t>Contatto: contratto API/OpenAPI di H-8b01 da congelare prima di PK-26.</t>
+          <t>HLS_* creata solo con autorizzazione esplicita (Q9); mai su collection esistenti.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="62" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>PK-26</t>
+          <t>PK-25</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Onda 4+ (dopo GO)</t>
+          <t>Onda 3+ (dopo GO)</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>UI (viste, permessi, grafica, npm) e sostituzione launcher</t>
+          <t>API loopback e read model</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>H-8b03, H-8b04, H-8b06, H-8b07, H-8b08</t>
+          <t>H-8b01, H-8b02, H-8b05</t>
         </is>
       </c>
       <c r="E37" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A37)+COUNTIF('Post-GO'!D5:D61,A37)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A37)+COUNTIF('Post-GO'!D5:D62,A37)</f>
         <v/>
       </c>
       <c r="F37" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A37,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A37,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A37,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A37,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G37" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A37,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A37,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F37=E37,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A37,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A37,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A37,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A37,'Post-GO'!I5:I61,"In review")+F37&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A37,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A37,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F37=E37,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A37,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A37,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A37,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A37,'Post-GO'!I5:I62,"In review")+F37&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>NARO</t>
+          <t>SCIBETTA</t>
         </is>
       </c>
       <c r="I37" s="9" t="inlineStr">
         <is>
-          <t>N13</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>T-8b06, T-405, T-8b07, T-8b09, T-8b10, T-304</t>
+          <t>T-8b01, T-8b04, T-8b05, T-8b08</t>
         </is>
       </c>
       <c r="K37" s="10" t="inlineStr">
         <is>
-          <t>ui/, [N] shim launcher :8799</t>
+          <t>api/</t>
         </is>
       </c>
       <c r="L37" s="10" t="inlineStr">
         <is>
-          <t>PK-25, PK-08, PK-06</t>
+          <t>GO; PK-06, PK-08</t>
         </is>
       </c>
       <c r="M37" s="10" t="inlineStr">
         <is>
-          <t>PK-25 (dopo contratto API)</t>
+          <t>PK-26 (dopo contratto API)</t>
         </is>
       </c>
       <c r="N37" s="10" t="inlineStr">
         <is>
-          <t>La UI non esegue build/test/git (C23–C24).</t>
+          <t>Contatto: contratto API/OpenAPI di H-8b01 da congelare prima di PK-26.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="62" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>PK-26b</t>
+          <t>PK-26</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -12227,24 +12343,24 @@
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Gate di configurazione all'avvio della dashboard</t>
+          <t>UI (viste, permessi, grafica, npm) e sostituzione launcher</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>H-8b09</t>
+          <t>H-8b03, H-8b04, H-8b06, H-8b07, H-8b08</t>
         </is>
       </c>
       <c r="E38" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A38)+COUNTIF('Post-GO'!D5:D61,A38)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A38)+COUNTIF('Post-GO'!D5:D62,A38)</f>
         <v/>
       </c>
       <c r="F38" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A38,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A38,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A38,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A38,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G38" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A38,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A38,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F38=E38,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A38,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A38,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A38,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A38,'Post-GO'!I5:I61,"In review")+F38&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A38,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A38,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F38=E38,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A38,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A38,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A38,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A38,'Post-GO'!I5:I62,"In review")+F38&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H38" s="9" t="inlineStr">
@@ -12254,66 +12370,66 @@
       </c>
       <c r="I38" s="9" t="inlineStr">
         <is>
-          <t>N13b</t>
+          <t>N13</t>
         </is>
       </c>
       <c r="J38" s="10" t="inlineStr">
         <is>
-          <t>T-8b11</t>
+          <t>T-8b06, T-405, T-8b07, T-8b09, T-8b10, T-304</t>
         </is>
       </c>
       <c r="K38" s="10" t="inlineStr">
         <is>
-          <t>api/ (gate), ui/ (dialog di prima configurazione)</t>
+          <t>ui/, [N] shim launcher :8799</t>
         </is>
       </c>
       <c r="L38" s="10" t="inlineStr">
         <is>
-          <t>PK-07b (H-309), PK-25 (H-8b01), PK-26 (H-8b03)</t>
+          <t>PK-25, PK-08, PK-06</t>
         </is>
       </c>
       <c r="M38" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PK-25 (dopo contratto API)</t>
         </is>
       </c>
       <c r="N38" s="10" t="inlineStr">
         <is>
-          <t>Il gate chiama il modulo di H-309: nessuna logica duplicata. Non aggirabile da chiamata diretta all'API (C23). Verifica: T-8b11, T-8b12, E2E-CFG-1.</t>
+          <t>La UI non esegue build/test/git (C23–C24).</t>
         </is>
       </c>
     </row>
     <row r="39" ht="62" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>PK-26c</t>
+          <t>PK-26b</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>Onda 5+ (dopo GO)</t>
+          <t>Onda 4+ (dopo GO)</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Pannello di avvio del run non presidiato</t>
+          <t>Gate di configurazione all'avvio della dashboard</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>H-8b10</t>
+          <t>H-8b09</t>
         </is>
       </c>
       <c r="E39" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A39)+COUNTIF('Post-GO'!D5:D61,A39)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A39)+COUNTIF('Post-GO'!D5:D62,A39)</f>
         <v/>
       </c>
       <c r="F39" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A39,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A39,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A39,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A39,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G39" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A39,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A39,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F39=E39,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A39,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A39,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A39,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A39,'Post-GO'!I5:I61,"In review")+F39&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A39,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A39,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F39=E39,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A39,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A39,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A39,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A39,'Post-GO'!I5:I62,"In review")+F39&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H39" s="9" t="inlineStr">
@@ -12323,22 +12439,22 @@
       </c>
       <c r="I39" s="9" t="inlineStr">
         <is>
-          <t>N13c</t>
+          <t>N13b</t>
         </is>
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>T-8b13, T-2</t>
+          <t>T-8b11</t>
         </is>
       </c>
       <c r="K39" s="10" t="inlineStr">
         <is>
-          <t>api/ (avvio run non presidiato), ui/ (pannello perimetro, limiti, kill switch)</t>
+          <t>api/ (gate), ui/ (dialog di prima configurazione)</t>
         </is>
       </c>
       <c r="L39" s="10" t="inlineStr">
         <is>
-          <t>PK-19b (H-713), PK-20b (H-714), PK-26 (H-8b03), PK-26b (H-8b09)</t>
+          <t>PK-07b (H-309), PK-25 (H-8b01), PK-26 (H-8b03)</t>
         </is>
       </c>
       <c r="M39" s="10" t="inlineStr">
@@ -12348,293 +12464,362 @@
       </c>
       <c r="N39" s="10" t="inlineStr">
         <is>
-          <t>C24: il run non presidiato lo avvia SEMPRE una sessione umana. Mostra perimetro e limiti prima dell'avvio; kill switch raggiungibile a run in corso. Verifica: T-8b13, E2E-AUT-2.</t>
+          <t>Il gate chiama il modulo di H-309: nessuna logica duplicata. Non aggirabile da chiamata diretta all'API (C23). Verifica: T-8b11, T-8b12, E2E-CFG-1.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="62" customHeight="1">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>PK-27</t>
+          <t>PK-26c</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Onda 7 (dopo GO)</t>
+          <t>Onda 5+ (dopo GO)</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Scenari E2E V1–V24</t>
+          <t>Pannello di avvio del run non presidiato</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>H-901</t>
+          <t>H-8b10</t>
         </is>
       </c>
       <c r="E40" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A40)+COUNTIF('Post-GO'!D5:D61,A40)</f>
+        <f>COUNTIF('Pre-GO'!D5:D26,A40)+COUNTIF('Post-GO'!D5:D62,A40)</f>
         <v/>
       </c>
       <c r="F40" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A40,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A40,'Post-GO'!I5:I61,"Fatto")</f>
+        <f>COUNTIFS('Pre-GO'!D5:D26,A40,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A40,'Post-GO'!I5:I62,"Fatto")</f>
         <v/>
       </c>
       <c r="G40" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A40,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A40,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F40=E40,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A40,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A40,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A40,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A40,'Post-GO'!I5:I61,"In review")+F40&gt;0,"In corso","Da fare")))</f>
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A40,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A40,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F40=E40,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A40,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A40,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A40,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A40,'Post-GO'!I5:I62,"In review")+F40&gt;0,"In corso","Da fare")))</f>
         <v/>
       </c>
       <c r="H40" s="9" t="inlineStr">
         <is>
-          <t>SCIBETTA</t>
+          <t>NARO</t>
         </is>
       </c>
       <c r="I40" s="9" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>N13c</t>
         </is>
       </c>
       <c r="J40" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>T-8b13, T-2</t>
         </is>
       </c>
       <c r="K40" s="10" t="inlineStr">
         <is>
-          <t>E2E_VERIFICATION.md, [N] repo pilota test\</t>
+          <t>api/ (avvio run non presidiato), ui/ (pannello perimetro, limiti, kill switch)</t>
         </is>
       </c>
       <c r="L40" s="10" t="inlineStr">
         <is>
-          <t>Fasi 5–8</t>
+          <t>PK-19b (H-713), PK-20b (H-714), PK-26 (H-8b03), PK-26b (H-8b09)</t>
         </is>
       </c>
       <c r="M40" s="10" t="inlineStr">
         <is>
-          <t>PK-28</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N40" s="10" t="inlineStr">
         <is>
-          <t>Esecuzione su 3 OS a cura del SUPERVISORE.</t>
+          <t>C24: il run non presidiato lo avvia SEMPRE una sessione umana. Mostra perimetro e limiti prima dell'avvio; kill switch raggiungibile a run in corso. Verifica: T-8b13, E2E-AUT-2.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="62" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
+          <t>PK-27</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Onda 7 (dopo GO)</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>Scenari E2E V1–V24</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>H-901</t>
+        </is>
+      </c>
+      <c r="E41" s="9">
+        <f>COUNTIF('Pre-GO'!D5:D26,A41)+COUNTIF('Post-GO'!D5:D62,A41)</f>
+        <v/>
+      </c>
+      <c r="F41" s="9">
+        <f>COUNTIFS('Pre-GO'!D5:D26,A41,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A41,'Post-GO'!I5:I62,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="G41" s="9">
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A41,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A41,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F41=E41,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A41,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A41,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A41,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A41,'Post-GO'!I5:I62,"In review")+F41&gt;0,"In corso","Da fare")))</f>
+        <v/>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>SCIBETTA</t>
+        </is>
+      </c>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="J41" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K41" s="10" t="inlineStr">
+        <is>
+          <t>E2E_VERIFICATION.md, [N] repo pilota test\</t>
+        </is>
+      </c>
+      <c r="L41" s="10" t="inlineStr">
+        <is>
+          <t>Fasi 5–8</t>
+        </is>
+      </c>
+      <c r="M41" s="10" t="inlineStr">
+        <is>
           <t>PK-28</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>Onda 7 (dopo GO)</t>
-        </is>
-      </c>
-      <c r="C41" s="10" t="inlineStr">
-        <is>
-          <t>README plugin e manuali</t>
-        </is>
-      </c>
-      <c r="D41" s="10" t="inlineStr">
-        <is>
-          <t>H-902, H-1101</t>
-        </is>
-      </c>
-      <c r="E41" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A41)+COUNTIF('Post-GO'!D5:D61,A41)</f>
-        <v/>
-      </c>
-      <c r="F41" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A41,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A41,'Post-GO'!I5:I61,"Fatto")</f>
-        <v/>
-      </c>
-      <c r="G41" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A41,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A41,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F41=E41,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A41,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A41,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A41,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A41,'Post-GO'!I5:I61,"In review")+F41&gt;0,"In corso","Da fare")))</f>
-        <v/>
-      </c>
-      <c r="H41" s="9" t="inlineStr">
-        <is>
-          <t>NARO</t>
-        </is>
-      </c>
-      <c r="I41" s="9" t="inlineStr">
-        <is>
-          <t>N14</t>
-        </is>
-      </c>
-      <c r="J41" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K41" s="10" t="inlineStr">
-        <is>
-          <t>agents/plugin/README.md, docs/ (manuali, NOTICE, runbook)</t>
-        </is>
-      </c>
-      <c r="L41" s="10" t="inlineStr">
-        <is>
-          <t>PK-27</t>
-        </is>
-      </c>
-      <c r="M41" s="10" t="inlineStr">
-        <is>
-          <t>PK-29</t>
-        </is>
-      </c>
       <c r="N41" s="10" t="inlineStr">
         <is>
-          <t>Revisione approvata dal SUPERVISORE.</t>
+          <t>Esecuzione su 3 OS a cura del SUPERVISORE.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="62" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
+          <t>PK-28</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Onda 7 (dopo GO)</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>README plugin e manuali</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>H-902, H-1101</t>
+        </is>
+      </c>
+      <c r="E42" s="9">
+        <f>COUNTIF('Pre-GO'!D5:D26,A42)+COUNTIF('Post-GO'!D5:D62,A42)</f>
+        <v/>
+      </c>
+      <c r="F42" s="9">
+        <f>COUNTIFS('Pre-GO'!D5:D26,A42,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A42,'Post-GO'!I5:I62,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="G42" s="9">
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A42,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A42,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F42=E42,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A42,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A42,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A42,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A42,'Post-GO'!I5:I62,"In review")+F42&gt;0,"In corso","Da fare")))</f>
+        <v/>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>NARO</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="inlineStr">
+        <is>
+          <t>N14</t>
+        </is>
+      </c>
+      <c r="J42" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K42" s="10" t="inlineStr">
+        <is>
+          <t>agents/plugin/README.md, docs/ (manuali, NOTICE, runbook)</t>
+        </is>
+      </c>
+      <c r="L42" s="10" t="inlineStr">
+        <is>
+          <t>PK-27</t>
+        </is>
+      </c>
+      <c r="M42" s="10" t="inlineStr">
+        <is>
           <t>PK-29</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
-        <is>
-          <t>Onda 8 (dopo GO)</t>
-        </is>
-      </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>Hardening</t>
-        </is>
-      </c>
-      <c r="D42" s="10" t="inlineStr">
-        <is>
-          <t>H-1001</t>
-        </is>
-      </c>
-      <c r="E42" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A42)+COUNTIF('Post-GO'!D5:D61,A42)</f>
-        <v/>
-      </c>
-      <c r="F42" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A42,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A42,'Post-GO'!I5:I61,"Fatto")</f>
-        <v/>
-      </c>
-      <c r="G42" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A42,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A42,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F42=E42,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A42,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A42,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A42,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A42,'Post-GO'!I5:I61,"In review")+F42&gt;0,"In corso","Da fare")))</f>
-        <v/>
-      </c>
-      <c r="H42" s="9" t="inlineStr">
-        <is>
-          <t>SCIBETTA</t>
-        </is>
-      </c>
-      <c r="I42" s="9" t="inlineStr">
-        <is>
-          <t>S14</t>
-        </is>
-      </c>
-      <c r="J42" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K42" s="10" t="inlineStr">
-        <is>
-          <t>[N] log immutabili, sandbox, SBOM</t>
-        </is>
-      </c>
-      <c r="L42" s="10" t="inlineStr">
-        <is>
-          <t>PK-27</t>
-        </is>
-      </c>
-      <c r="M42" s="10" t="inlineStr">
-        <is>
-          <t>PK-28</t>
-        </is>
-      </c>
       <c r="N42" s="10" t="inlineStr">
         <is>
-          <t>[N] nessun T-xxx in IN §6: verifica = audit.</t>
+          <t>Revisione approvata dal SUPERVISORE.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="62" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
+          <t>PK-29</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Onda 8 (dopo GO)</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Hardening</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>H-1001</t>
+        </is>
+      </c>
+      <c r="E43" s="9">
+        <f>COUNTIF('Pre-GO'!D5:D26,A43)+COUNTIF('Post-GO'!D5:D62,A43)</f>
+        <v/>
+      </c>
+      <c r="F43" s="9">
+        <f>COUNTIFS('Pre-GO'!D5:D26,A43,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A43,'Post-GO'!I5:I62,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="G43" s="9">
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A43,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A43,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F43=E43,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A43,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A43,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A43,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A43,'Post-GO'!I5:I62,"In review")+F43&gt;0,"In corso","Da fare")))</f>
+        <v/>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>SCIBETTA</t>
+        </is>
+      </c>
+      <c r="I43" s="9" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="J43" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K43" s="10" t="inlineStr">
+        <is>
+          <t>[N] log immutabili, sandbox, SBOM</t>
+        </is>
+      </c>
+      <c r="L43" s="10" t="inlineStr">
+        <is>
+          <t>PK-27</t>
+        </is>
+      </c>
+      <c r="M43" s="10" t="inlineStr">
+        <is>
+          <t>PK-28</t>
+        </is>
+      </c>
+      <c r="N43" s="10" t="inlineStr">
+        <is>
+          <t>[N] nessun T-xxx in IN §6: verifica = audit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="62" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
           <t>PK-30</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>Onda 9 (dopo GO)</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
         <is>
           <t>Rollout sul pilota</t>
         </is>
       </c>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="D44" s="10" t="inlineStr">
         <is>
           <t>H-1201</t>
         </is>
       </c>
-      <c r="E43" s="9">
-        <f>COUNTIF('Pre-GO'!D5:D26,A43)+COUNTIF('Post-GO'!D5:D61,A43)</f>
-        <v/>
-      </c>
-      <c r="F43" s="9">
-        <f>COUNTIFS('Pre-GO'!D5:D26,A43,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D61,A43,'Post-GO'!I5:I61,"Fatto")</f>
-        <v/>
-      </c>
-      <c r="G43" s="9">
-        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A43,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D61,A43,'Post-GO'!I5:I61,"Bloccato")&gt;0,"Bloccato",IF(F43=E43,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A43,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D61,A43,'Post-GO'!I5:I61,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A43,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D61,A43,'Post-GO'!I5:I61,"In review")+F43&gt;0,"In corso","Da fare")))</f>
-        <v/>
-      </c>
-      <c r="H43" s="9" t="inlineStr">
+      <c r="E44" s="9">
+        <f>COUNTIF('Pre-GO'!D5:D26,A44)+COUNTIF('Post-GO'!D5:D62,A44)</f>
+        <v/>
+      </c>
+      <c r="F44" s="9">
+        <f>COUNTIFS('Pre-GO'!D5:D26,A44,'Pre-GO'!I5:I26,"Fatto")+COUNTIFS('Post-GO'!D5:D62,A44,'Post-GO'!I5:I62,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="G44" s="9">
+        <f>IF(COUNTIFS('Pre-GO'!D5:D26,A44,'Pre-GO'!I5:I26,"Bloccato")+COUNTIFS('Post-GO'!D5:D62,A44,'Post-GO'!I5:I62,"Bloccato")&gt;0,"Bloccato",IF(F44=E44,"Fatto",IF(COUNTIFS('Pre-GO'!D5:D26,A44,'Pre-GO'!I5:I26,"In corso")+COUNTIFS('Post-GO'!D5:D62,A44,'Post-GO'!I5:I62,"In corso")+COUNTIFS('Pre-GO'!D5:D26,A44,'Pre-GO'!I5:I26,"In review")+COUNTIFS('Post-GO'!D5:D62,A44,'Post-GO'!I5:I62,"In review")+F44&gt;0,"In corso","Da fare")))</f>
+        <v/>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
         <is>
           <t>NARO</t>
         </is>
       </c>
-      <c r="I43" s="9" t="inlineStr">
+      <c r="I44" s="9" t="inlineStr">
         <is>
           <t>N15</t>
         </is>
       </c>
-      <c r="J43" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K43" s="10" t="inlineStr">
+      <c r="J44" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K44" s="10" t="inlineStr">
         <is>
           <t>docs/ (metriche, rollback)</t>
         </is>
       </c>
-      <c r="L43" s="10" t="inlineStr">
+      <c r="L44" s="10" t="inlineStr">
         <is>
           <t>PK-28, PK-29</t>
         </is>
       </c>
-      <c r="M43" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N43" s="10" t="inlineStr">
+      <c r="M44" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N44" s="10" t="inlineStr">
         <is>
           <t>[N] parere legale; pilota da scegliere.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N43"/>
+  <autoFilter ref="A4:N44"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G43">
+  <conditionalFormatting sqref="G5:G44">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"Fatto"</formula>
     </cfRule>
@@ -12648,7 +12833,7 @@
       <formula>"Da fare"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H43">
+  <conditionalFormatting sqref="H5:H44">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
       <formula>"NARO"</formula>
     </cfRule>

</xml_diff>